<commit_message>
chore: Update song list to Jul.28, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -16145,7 +16145,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I390" t="inlineStr"/>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>BV1HYgy6REZM</t>
+        </is>
+      </c>
       <c r="J390" t="inlineStr"/>
     </row>
     <row r="391">
@@ -16413,7 +16417,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I397" t="inlineStr"/>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>BV1pagy6xEgX</t>
+        </is>
+      </c>
       <c r="J397" t="inlineStr"/>
     </row>
     <row r="398">
@@ -23469,7 +23477,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I577" t="inlineStr"/>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>BV1zzuKzpEc5</t>
+        </is>
+      </c>
       <c r="J577" t="inlineStr"/>
     </row>
     <row r="578">
@@ -23585,7 +23597,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I580" t="inlineStr"/>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>BV1GbgX68EMy</t>
+        </is>
+      </c>
       <c r="J580" t="inlineStr"/>
     </row>
     <row r="581">
@@ -24389,7 +24405,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I601" t="inlineStr"/>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>BV1Qx3w6pEUx</t>
+        </is>
+      </c>
       <c r="J601" t="inlineStr"/>
     </row>
     <row r="602">
@@ -24425,7 +24445,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I602" t="inlineStr"/>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>BV1DDgk6eEWB</t>
+        </is>
+      </c>
       <c r="J602" t="inlineStr"/>
     </row>
     <row r="603">
@@ -35253,7 +35277,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="I877" t="inlineStr"/>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>BV19x3P6cEPV</t>
+        </is>
+      </c>
       <c r="J877" t="inlineStr"/>
     </row>
     <row r="878">
@@ -35289,7 +35317,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I878" t="inlineStr"/>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>BV1Xx3P6cEfK</t>
+        </is>
+      </c>
       <c r="J878" t="inlineStr"/>
     </row>
     <row r="879">
@@ -35325,7 +35357,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I879" t="inlineStr"/>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>BV1D43w6QE1L</t>
+        </is>
+      </c>
       <c r="J879" t="inlineStr"/>
     </row>
     <row r="880">
@@ -35361,7 +35397,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I880" t="inlineStr"/>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>BV1CU3B6VEPC</t>
+        </is>
+      </c>
       <c r="J880" t="inlineStr"/>
     </row>
     <row r="881">
@@ -35397,7 +35437,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I881" t="inlineStr"/>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>BV19x3P6cENj</t>
+        </is>
+      </c>
       <c r="J881" t="inlineStr"/>
     </row>
     <row r="882">
@@ -35433,7 +35477,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I882" t="inlineStr"/>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>BV1g8gX6fEqx</t>
+        </is>
+      </c>
       <c r="J882" t="inlineStr"/>
     </row>
     <row r="883">
@@ -35469,7 +35517,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I883" t="inlineStr"/>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>BV19x3P6cESt</t>
+        </is>
+      </c>
       <c r="J883" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: Update song list to Aug.16, 2026
</commit_message>
<xml_diff>
--- a/scripts/Book1.xlsx
+++ b/scripts/Book1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J883"/>
+  <dimension ref="A1:J889"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -539,7 +539,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/09，2025/11/14，2025/12/24，2025/12/26，2026/01/16，2026/01/24，2026/01/28，2026/01/30，2026/02/10，2026/02/14，2026/03/09，2026/03/27，2026/04/01，2026/04/14，2026/04/24，2026/06/12，2026/07/22</t>
+          <t>2025/03/01，2025/03/15，2025/04/01，2025/04/15，2025/04/26，2025/05/09，2025/05/30，2025/06/08，2025/07/05，2025/07/11，2025/08/13，2025/09/17，2025/09/02，2025/09/07，2025/09/19，2025/10/01，2025/10/09，2025/10/16，2025/10/24，2025/10/30，2025/11/09，2025/11/14，2025/12/24，2025/12/26，2026/01/16，2026/01/24，2026/01/28，2026/01/30，2026/02/10，2026/02/14，2026/03/09，2026/03/27，2026/04/01，2026/04/14，2026/04/24，2026/06/12，2026/07/22，2026/08/11</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -550,7 +550,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/07，2026/01/14，2026/01/24，2026/02/19，2026/03/07，2026/03/15，2026/06/06，2026/06/23</t>
+          <t>2025/03/02，2025/03/29，2025/05/06，2025/05/30，2025/06/28，2025/09/04，2025/09/18，2025/11/07，2026/01/14，2026/01/24，2026/02/19，2026/03/07，2026/03/15，2026/06/06，2026/06/23，2026/08/05，2026/08/05</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -594,7 +594,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19</t>
+          <t>2025/03/02，2025/03/29，2025/04/11，2025/04/17，2025/04/26，2025/05/04，2025/05/09，2025/05/17，2025/05/24，2025/06/02，2025/06/20，2025/06/27，2025/07/11，2025/07/21，2025/07/26，2025/08/08，2025/08/29，2025/09/02，2025/10/03，2025/10/09，2025/10/22，2025/11/09，2025/12/11，2026/01/15，2026/02/12，2026/04/19，2026/08/08</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -686,7 +686,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/01，2025/11/17，2025/12/02，2025/12/31，2026/02/02，2026/02/14，2026/03/06，2026/04/01，2026/04/20，2026/05/15，2026/06/10，2026/07/22</t>
+          <t>2025/03/02，2025/03/14，2025/03/28，2025/04/17，2025/04/25，2025/05/12，2025/05/12，2025/05/18，2025/05/29，2025/06/02，2025/06/05，2025/06/12，2025/06/27，2025/07/10，2025/08/04，2025/08/08，2025/08/21，2025/08/28，2025/09/10，2025/09/22，2025/09/30，2025/10/12，2025/11/01，2025/11/17，2025/12/02，2025/12/31，2026/02/02，2026/02/14，2026/03/06，2026/04/01，2026/04/20，2026/05/15，2026/06/10，2026/07/22，2026/08/09</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -726,7 +726,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/09，2025/11/19，2025/12/16，2026/01/16，2026/01/28，2026/02/07，2026/02/10，2026/03/17，2026/04/19，2026/05/23，2026/06/19，2026/07/22</t>
+          <t>2025/03/03，2025/03/21，2025/04/17，2025/04/21，2025/05/12，2025/05/26，2025/05/30，2025/06/26，2025/07/07，2025/07/13，2025/07/26，2025/08/12，2025/08/22，2025/09/19，2025/10/03，2025/10/28，2025/11/09，2025/11/19，2025/12/16，2026/01/16，2026/01/28，2026/02/07，2026/02/10，2026/03/17，2026/04/19，2026/05/23，2026/06/19，2026/07/22，2026/08/08</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -770,7 +770,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/04/04，2025/04/14，2025/04/20，2025/04/24，2025/05/09，2025/05/18，2025/05/29，2025/06/06，2025/08/01，2025/09/21，2025/10/10，2025/11/28，2025/12/08，2025/12/30，2026/04/26，2026/07/09</t>
+          <t>2025/03/03，2025/04/04，2025/04/14，2025/04/20，2025/04/24，2025/05/09，2025/05/18，2025/05/29，2025/06/06，2025/08/01，2025/09/21，2025/10/10，2025/11/28，2025/12/08，2025/12/30，2026/04/26，2026/07/09，2026/07/31</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -850,7 +850,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/07，2025/12/31，2026/01/14，2026/01/19，2026/03/29，2026/04/12，2026/04/27，2026/05/01，2026/06/03，2026/06/18，2026/06/25</t>
+          <t>2025/03/03，2025/03/25，2025/04/03，2025/04/07，2025/04/18，2025/04/24，2025/05/04，2025/05/12，2025/05/16，2025/05/19，2025/05/30，2025/06/02，2025/06/09，2025/06/13，2025/07/05，2025/07/14，2025/07/21，2025/07/28，2025/08/29，2025/09/04，2025/09/07，2025/10/05，2025/10/10，2025/10/22，2025/11/10，2025/12/07，2025/12/31，2026/01/14，2026/01/19，2026/03/29，2026/04/12，2026/04/27，2026/05/01，2026/06/03，2026/06/18，2026/06/25，2026/07/31</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -930,7 +930,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/01/03，2026/03/25，2026/05/10，2026/06/20</t>
+          <t>2025/03/04，2025/03/30，2025/05/01，2025/05/26，2025/06/17，2025/08/03，2025/09/26，2025/10/26，2026/01/03，2026/03/25，2026/05/10，2026/06/20，2026/8/16</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/04/07，2025/05/29，2025/06/06，2025/06/19，2025/06/26，2025/07/10，2025/07/11，2025/07/14，2025/08/02，2025/09/03，2025/09/26，2025/10/03，2025/11/09，2025/11/24，2025/11/26，2026/01/05，2026/01/30，2026/03/04，2026/06/17</t>
+          <t>2025/03/04，2025/04/07，2025/05/29，2025/06/06，2025/06/19，2025/06/26，2025/07/10，2025/07/11，2025/07/14，2025/08/02，2025/09/03，2025/09/26，2025/10/03，2025/11/09，2025/11/24，2025/11/26，2026/01/05，2026/01/30，2026/03/04，2026/06/17，2026/08/05</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/09，2025/12/30，2026/02/20，2026/02/23，2026/03/04，2026/04/11，2026/04/16，2026/04/23，2026/06/14，2026/07/04</t>
+          <t>2025/03/04，2025/03/14，2025/04/15，2025/05/03，2025/05/19，2025/07/18，2025/07/28，2025/08/28，2025/09/22，2025/10/19，2025/10/26，2025/11/09，2025/12/30，2026/02/20，2026/02/23，2026/03/04，2026/04/11，2026/04/16，2026/04/23，2026/06/14，2026/07/04，2026/07/31</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/01，2025/11/09，2025/11/21，2025/12/08，2026/01/15，2026/01/24，2026/03/04，2026/03/14，2026/05/06，2026/05/16，2026/05/20，2026/06/12，2026/07/16，2026/07/26</t>
+          <t>2025/03/04，2025/03/13，2025/04/03，2025/05/12，2025/05/19，2025/05/23，2025/05/25，2025/06/12，2025/07/15，2025/07/20，2025/07/23，2025/08/02，2025/08/10，2025/08/29，2025/09/17，2025/09/19，2025/09/27，2025/10/22，2025/11/01，2025/11/09，2025/11/21，2025/12/08，2026/01/15，2026/01/24，2026/03/04，2026/03/14，2026/05/06，2026/05/16，2026/05/20，2026/06/12，2026/07/16，2026/07/26，2026/07/31</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/01，2025/11/28，2025/12/12，2026/01/05，2026/01/22，2026/03/04，2026/03/08，2026/03/22，2026/04/22，2026/04/24，2026/05/10，2026/05/23，2026/06/10，2026/06/15</t>
+          <t>2025/03/04，2025/03/30，2025/04/14，2025/04/25，2025/06/05，2025/06/13，2025/06/26，2025/07/13，2025/07/24，2025/08/12，2025/08/28，2025/09/26，2025/10/07，2025/10/11，2025/11/01，2025/11/28，2025/12/12，2026/01/05，2026/01/22，2026/03/04，2026/03/08，2026/03/22，2026/04/22，2026/04/24，2026/05/10，2026/05/23，2026/06/10，2026/06/15，2026/07/31，2026/08/11</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/07，2025/12/24，2026/01/01，2026/01/16，2026/03/14，2026/05/01，2026/05/20</t>
+          <t>2025/03/04，2025/03/14，2025/04/17，2025/05/06，2025/05/25，2025/05/25，2025/05/31，2025/09/03，2025/11/07，2025/12/24，2026/01/01，2026/01/16，2026/03/14，2026/05/01，2026/05/20，2026/08/01</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/01/14，2026/02/19，2026/03/14，2026/04/16，2026/06/17，2026/07/16，2026/07/22</t>
+          <t>2025/03/06，2025/03/20，2025/04/02，2025/04/10，2025/04/19，2025/04/27，2025/05/13，2025/05/15，2025/05/18，2025/05/26，2025/06/06，2025/06/12，2025/06/21，2025/07/05，2025/07/10，2025/07/13，2025/07/27，2025/08/29，2025/09/13，2025/09/19，2025/09/28，2025/10/23，2025/10/28，2025/12/23，2026/01/14，2026/02/19，2026/03/14，2026/04/16，2026/06/17，2026/07/16，2026/07/22，2026/08/11</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2134,7 +2134,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05</t>
+          <t>2025/03/06，2025/03/19，2025/04/11，2025/05/03，2025/07/10，2025/09/05，2025/09/18，2025/10/01，2025/11/07，2025/11/09，2025/12/02，2026/01/21，2026/03/05，2026/04/16，2026/06/23，2026/07/05，2026/08/05，2026/08/05</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/03，2025/12/12，2026/02/04，2026/04/18，2026/05/20，2026/06/20</t>
+          <t>2025/03/06，2025/04/13，2025/05/01，2025/06/15，2025/07/24，2025/08/30，2025/09/05，2025/10/09，2025/11/03，2025/12/12，2026/02/04，2026/04/18，2026/05/20，2026/06/20，2026/07/30，2026/08/09</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2795,7 +2795,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/01，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/01/09，2026/01/22，2026/02/14，2026/03/22，2026/04/19，2026/05/01，2026/05/23，2026/06/25</t>
+          <t>2025/03/07，2025/03/28，2025/04/24，2025/04/27，2025/05/01，2025/05/23，2025/05/25，2025/06/23，2025/07/03，2025/07/20，2025/07/27，2025/08/19，2025/09/06，2025/09/21，2025/10/17，2025/10/19，2025/11/01，2025/11/10，2025/11/18，2025/11/24，2025/12/23，2026/01/09，2026/01/22，2026/02/14，2026/03/22，2026/04/19，2026/05/01，2026/05/23，2026/06/25，2026/08/07</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20</t>
+          <t>2025/03/07，2025/03/21，2025/04/04，2025/04/18，2025/04/29，2025/05/08，2025/05/22，2025/05/25，2025/06/06，2025/06/08，2025/06/13，2025/06/13，2025/06/26，2025/07/03，2025/07/05，2025/07/11，2025/07/14，2025/07/26，2025/08/02，2025/08/12，2025/08/21，2025/09/17，2025/11/01，2025/11/09，2025/12/04，2025/12/16，2025/12/31，2026/01/09，2026/01/15，2026/01/21，2026/01/23，2026/01/29，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/02/24，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/05，2026/03/07，2026/03/08，2026/03/09，2026/03/12，2026/03/13，2026/03/14，2026/03/15，2026/03/17，2026/03/18，2026/03/19，2026/03/22，2026/03/24，2026/03/27，2026/03/28，2026/03/31，2026/04/08，2026/04/14，2026/04/18，2026/04/25，2026/05/01，2026/05/15，2026/05/25，2026/06/12，2026/06/23，2026/06/26，2026/07/04，2026/07/20，2026/07/30，2026/08/09</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>72</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2025/03/07，2025/04/11，2025/04/29，2025/08/01，2025/10/26，2026/02/19，2026/02/23，2026/03/06</t>
+          <t>2025/03/07，2025/04/11，2025/04/29，2025/08/01，2025/10/26，2026/02/19，2026/02/23，2026/03/06，2026/08/02</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/01，2026/01/16，2026/02/02，2026/02/23，2026/03/08，2026/03/19，2026/03/21，2026/04/16，2026/05/10，2026/06/14，2026/07/25</t>
+          <t>2025/03/09，2025/03/14，2025/04/07，2025/04/15，2025/04/27，2025/05/12，2025/05/27，2025/06/05，2025/06/08，2025/07/20，2025/08/01，2025/09/21，2025/09/28，2025/10/07，2025/10/18，2025/10/24，2025/11/10，2025/12/01，2026/01/16，2026/02/02，2026/02/23，2026/03/08，2026/03/19，2026/03/21，2026/04/16，2026/05/10，2026/06/14，2026/07/25，2026/08/07</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/09，2026/01/01，2026/06/20</t>
+          <t>2025/03/09，2025/03/30，2025/04/10，2025/04/20，2025/05/04，2025/05/13，2025/05/22，2025/06/05，2025/06/07，2025/08/29，2025/09/07，2025/09/11，2025/10/10，2025/11/09，2026/01/01，2026/06/20，2026/07/30</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/03/27，2026/04/01，2026/06/23</t>
+          <t>2025/03/10，2025/03/14，2025/05/09，2025/06/03，2025/07/18，2025/07/22，2025/08/28，2025/09/30，2025/11/27，2026/03/27，2026/04/01，2026/06/23，2026/07/31</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/01/01，2026/02/14，2026/05/06，2026/05/23，2026/07/07</t>
+          <t>2025/03/12，2025/04/29，2025/06/02，2025/09/21，2025/10/07，2025/10/28，2025/12/13，2026/01/01，2026/02/14，2026/05/06，2026/05/23，2026/07/07，2026/08/02</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/04，2025/11/07，2025/11/09，2025/12/04，2026/01/09，2026/01/19，2026/01/21，2026/01/25，2026/03/04，2026/03/07，2026/03/14，2026/06/06，2026/06/19</t>
+          <t>2025/03/12，2025/04/04，2025/04/19，2025/04/26，2025/06/03，2025/06/19，2025/06/26，2025/07/10，2025/07/17，2025/07/31，2025/08/24，2025/08/30，2025/09/13，2025/09/18，2025/09/19，2025/09/22，2025/09/27，2025/10/01，2025/10/24，2025/10/31，2025/11/04，2025/11/07，2025/11/09，2025/12/04，2026/01/09，2026/01/19，2026/01/21，2026/01/25，2026/03/04，2026/03/07，2026/03/14，2026/06/06，2026/06/19，2026/08/05，2026/08/05</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -3886,7 +3886,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>35</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/03，2025/12/02，2025/12/04，2025/12/12，2026/01/05，2026/01/14，2026/02/19，2026/03/04，2026/03/31，2026/04/12，2026/04/29，2026/05/15，2026/06/12，2026/06/23，2026/07/09</t>
+          <t>2025/03/12，2025/04/07，2025/04/18，2025/05/10，2025/05/15，2025/05/29，2025/06/03，2025/06/16，2025/07/08，2025/07/08，2025/08/01，2025/09/04，2025/09/28，2025/10/25，2025/10/28，2025/11/03，2025/12/02，2025/12/04，2025/12/12，2026/01/05，2026/01/14，2026/02/19，2026/03/04，2026/03/31，2026/04/12，2026/04/29，2026/05/15，2026/06/12，2026/06/23，2026/07/09，2026/08/11</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -3934,7 +3934,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -4327,7 +4327,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2025/03/13，2025/04/13，2025/04/19，2025/05/06，2025/06/03，2025/08/28，2025/09/17，2025/10/10，2025/11/17，2025/11/22，2025/12/24，2026/01/15，2026/01/29，2026/03/19，2026/05/15</t>
+          <t>2025/03/13，2025/04/13，2025/04/19，2025/05/06，2025/06/03，2025/08/28，2025/09/17，2025/10/10，2025/11/17，2025/11/22，2025/12/24，2026/01/15，2026/01/29，2026/03/19，2026/05/15，2026/08/08</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4338,7 +4338,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/05/20，2025/07/23，2025/11/28，2025/12/09</t>
+          <t>2025/03/14，2025/05/20，2025/07/23，2025/11/28，2025/12/09，2026/07/31</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/09，2026/01/15，2026/02/19，2026/03/13，2026/03/15，2026/03/21，2026/06/14，2026/06/17，2026/07/20</t>
+          <t>2025/03/14，2025/04/02，2025/05/10，2025/05/18，2025/05/23，2025/06/05，2025/06/08，2025/06/27，2025/09/03，2025/09/21，2025/10/30，2025/11/22，2025/12/09，2026/01/15，2026/02/19，2026/03/13，2026/03/15，2026/03/21，2026/06/14，2026/06/17，2026/07/20，2026/07/31</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/01/02，2026/01/30，2026/04/09</t>
+          <t>2025/03/14，2025/03/28，2025/04/18，2025/09/20，2025/10/12，2025/10/22，2026/01/02，2026/01/30，2026/04/09，2026/07/31</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5230,7 +5230,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/03，2025/11/24，2026/04/09，2026/04/14，2026/04/24，2026/05/23</t>
+          <t>2025/03/14，2025/04/24，2025/05/25，2025/08/21，2025/09/10，2025/11/03，2025/11/24，2026/04/09，2026/04/14，2026/04/24，2026/05/23，2026/08/02</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5270,7 +5270,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -5299,7 +5299,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2025/03/14，2025/04/12，2025/05/20，2025/05/30，2025/06/27，2025/08/13，2025/09/11，2025/10/28，2025/12/20，2026/01/16，2026/04/17</t>
+          <t>2025/03/14，2025/04/12，2025/05/20，2025/05/30，2025/06/27，2025/08/13，2025/09/11，2025/10/28，2025/12/20，2026/01/16，2026/04/17，2026/08/08</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5310,7 +5310,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2025/03/15，2025/05/22，2025/06/10，2025/11/09，2025/11/14，2026/03/19，2026/06/15</t>
+          <t>2025/03/15，2025/05/22，2025/06/10，2025/11/09，2025/11/14，2026/03/19，2026/06/15，2026/08/02</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -5590,7 +5590,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21</t>
+          <t>2025/03/17，2025/03/28，2025/04/15，2025/04/19，2025/04/25，2025/05/01，2025/05/18，2025/05/25，2025/05/29，2025/06/05，2025/06/12，2025/06/22，2025/07/03，2025/07/11，2025/07/18，2025/07/22，2025/07/31，2025/08/01，2025/08/02，2025/08/03，2025/08/12，2025/09/03，2025/09/11，2025/09/18，2025/09/26，2025/10/03，2025/10/09，2025/10/20，2025/11/12，2025/12/07，2025/12/23，2026/01/05，2026/01/21，2026/01/29，2026/02/09，2026/02/20，2026/02/23，2026/03/04，2026/03/06，2026/03/07，2026/04/11，2026/04/14，2026/04/29，2026/05/23，2026/07/03，2026/07/21，2026/08/11</t>
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/03/27，2025/04/25，2025/05/01，2025/05/15，2025/06/10，2025/07/03，2025/09/11，2025/12/11，2026/01/09</t>
+          <t>2025/03/17，2025/03/27，2025/04/25，2025/05/01，2025/05/15，2025/06/10，2025/07/03，2025/09/11，2025/12/11，2026/01/09，2026/08/11</t>
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/17，2025/05/13，2025/05/23，2025/07/21，2025/07/29，2025/08/07，2025/09/30，2025/10/31，2025/12/09，2026/01/12，2026/04/26，2026/07/09</t>
+          <t>2025/03/17，2025/04/17，2025/05/13，2025/05/23，2025/07/21，2025/07/29，2025/08/07，2025/09/30，2025/10/31，2025/12/09，2026/01/12，2026/04/26，2026/07/09，2026/08/02</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/05/17，2025/06/01，2025/09/21，2025/10/09，2025/11/26</t>
+          <t>2025/03/17，2025/05/17，2025/06/01，2025/09/21，2025/10/09，2025/11/26，2026/08/02</t>
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
@@ -5950,7 +5950,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/09，2026/04/26</t>
+          <t>2025/03/17，2025/04/29，2025/06/03，2025/07/24，2025/08/01，2025/08/03，2025/10/10，2025/11/09，2026/04/26，2026/08/02</t>
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
@@ -6030,7 +6030,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/12，2025/09/02，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15</t>
+          <t>2025/03/17，2025/06/05，2025/06/05，2025/06/23，2025/08/12，2025/09/12，2025/09/02，2025/11/09，2025/12/04，2026/01/01，2026/01/29，2026/04/09，2026/06/15，2026/08/05</t>
         </is>
       </c>
       <c r="F138" t="inlineStr"/>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09</t>
+          <t>2025/03/18，2025/03/25，2025/04/02，2025/04/17，2025/05/01，2025/05/08，2025/05/10，2025/05/24，2025/05/29，2025/06/23，2025/06/27，2025/07/08，2025/07/28，2025/08/03，2025/09/08，2025/09/22，2025/10/03，2025/10/11，2025/10/16，2025/10/24，2025/11/18，2025/12/02，2025/12/17，2026/01/09，2026/01/15，2026/02/02，2026/02/14，2026/03/13，2026/03/25，2026/04/24，2026/05/23，2026/06/17，2026/07/05，2026/07/09，2026/07/31，2026/08/08</t>
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>36</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -6139,7 +6139,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2025/03/18，2025/03/25，2025/05/22，2025/07/10，2025/09/08，2025/10/09，2025/11/01，2026/01/15，2026/04/08</t>
+          <t>2025/03/18，2025/03/25，2025/05/22，2025/07/10，2025/09/08，2025/10/09，2025/11/01，2026/01/15，2026/04/08，2026/8/16</t>
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/01/03，2026/01/05，2026/01/30，2026/03/14，2026/03/31，2026/04/20，2026/05/01，2026/06/19，2026/06/30，2026/07/18</t>
+          <t>2025/03/19，2025/04/07，2025/04/21，2025/05/01，2025/05/10，2025/05/27，2025/06/09，2025/06/23，2025/06/26，2025/07/03，2025/09/15，2025/09/28，2025/10/01，2025/10/17，2026/01/03，2026/01/05，2026/01/30，2026/03/14，2026/03/31，2026/04/20，2026/05/01，2026/06/19，2026/06/30，2026/07/18，2026/08/03</t>
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/01/02，2026/01/15，2026/01/28，2026/02/19，2026/03/05，2026/04/09，2026/06/06，2026/06/20</t>
+          <t>2025/03/19，2025/07/07，2025/08/12，2025/08/26，2025/09/13，2025/09/17，2025/10/10，2025/11/21，2025/12/11，2026/01/02，2026/01/15，2026/01/28，2026/02/19，2026/03/05，2026/04/09，2026/06/06，2026/06/20，2026/07/31，2026/07/31</t>
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/04/11，2025/05/19，2025/05/23，2025/06/12，2025/06/23，2025/07/20，2025/08/19，2025/09/21，2025/10/07，2025/10/20，2025/10/28，2025/11/09，2025/11/24，2025/12/16，2025/12/24，2025/12/26，2026/05/23</t>
+          <t>2025/03/19，2025/03/28，2025/04/11，2025/05/19，2025/05/23，2025/06/12，2025/06/23，2025/07/20，2025/08/19，2025/09/21，2025/10/07，2025/10/20，2025/10/28，2025/11/09，2025/11/24，2025/12/16，2025/12/24，2025/12/26，2026/05/23，2026/07/30</t>
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
@@ -6390,7 +6390,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -6499,7 +6499,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19</t>
+          <t>2025/03/19，2025/03/28，2025/03/29，2025/04/11，2025/05/08，2025/05/22，2025/05/25，2025/05/29，2025/06/15，2025/07/14，2025/08/21，2025/09/26，2025/10/03，2025/11/19，2025/11/26，2026/01/01，2026/01/09，2026/03/22，2026/04/09，2026/04/20，2026/05/25，2026/06/10，2026/06/19，2026/08/11</t>
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/06/03</t>
+          <t>2025/03/20，2025/06/03，2026/8/16</t>
         </is>
       </c>
       <c r="F151" t="inlineStr"/>
@@ -6590,7 +6590,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/08，2025/12/24，2026/01/28，2026/04/22，2026/05/05，2026/06/14，2026/07/22</t>
+          <t>2025/03/20，2025/04/04，2025/04/17，2025/04/21，2025/04/29，2025/05/08，2025/05/30，2025/06/13，2025/06/26，2025/07/08，2025/07/18，2025/08/22，2025/09/05，2025/09/28，2025/10/25，2025/11/10，2025/11/27，2025/12/08，2025/12/24，2026/01/28，2026/04/22，2026/05/05，2026/06/14，2026/07/22，2026/07/31</t>
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
@@ -6634,7 +6634,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/19，2025/06/08，2025/06/12，2025/07/13，2025/08/28，2025/09/26，2025/10/25，2025/11/19，2025/11/27，2026/01/22，2026/01/25，2026/02/19，2026/05/20，2026/07/02</t>
+          <t>2025/03/20，2025/04/04，2025/05/19，2025/06/08，2025/06/12，2025/07/13，2025/08/28，2025/09/26，2025/10/25，2025/11/19，2025/11/27，2026/01/22，2026/01/25，2026/02/19，2026/05/20，2026/07/02，2026/08/02，2026/08/09</t>
         </is>
       </c>
       <c r="F154" t="inlineStr"/>
@@ -6714,7 +6714,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -6823,7 +6823,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04</t>
+          <t>2025/03/20，2025/04/04，2025/05/03，2025/05/22，2025/06/05，2025/07/25，2025/08/26，2025/08/16，2025/09/21，2025/10/03，2025/11/12，2025/12/08，2026/01/23，2026/01/26，2026/02/07，2026/02/10，2026/02/23，2026/02/25，2026/02/27，2026/03/01，2026/03/04，2026/03/13，2026/03/24，2026/03/28，2026/03/29，2026/04/27，2026/05/02，2026/06/18，2026/07/04，2026/07/31</t>
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -6947,7 +6947,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/06/26，2026/04/14，2026/06/10</t>
+          <t>2025/03/20，2025/06/26，2026/04/14，2026/06/10，2026/08/02</t>
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/01/16，2026/02/07，2026/03/28</t>
+          <t>2025/03/20，2025/04/17，2025/05/01，2025/05/03，2025/05/18，2025/05/22，2025/05/29，2025/06/06，2025/06/13，2025/06/30，2025/07/09，2025/07/27，2025/08/23，2025/09/03，2025/09/11，2025/10/11，2025/10/17，2025/12/24，2026/01/16，2026/02/07，2026/03/28，2026/8/16</t>
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>2025/03/21，2026/06/12</t>
+          <t>2025/03/21，2026/06/12，2026/08/02</t>
         </is>
       </c>
       <c r="F165" t="inlineStr"/>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09</t>
+          <t>2025/03/21，2025/04/06，2025/04/18，2025/04/25，2025/05/27，2025/07/11，2025/07/24，2025/08/09，2025/09/15，2025/09/21，2025/10/11，2025/10/24，2025/11/03，2025/11/22，2026/01/22，2026/02/19，2026/03/15，2026/04/02，2026/05/01，2026/05/23，2026/07/09，2026/08/11</t>
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
@@ -7550,7 +7550,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17</t>
+          <t>2025/03/21，2025/05/09，2025/05/30，2025/07/22，2025/09/28，2025/11/18，2025/12/08，2026/02/18，2026/03/06，2026/03/13，2026/03/14，2026/03/31，2026/05/01，2026/06/28，2026/07/17，2026/08/02</t>
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
@@ -7634,7 +7634,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -7827,7 +7827,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>2025/03/21，2025/04/28，2025/05/13，2025/06/07，2025/06/21，2025/08/28，2025/09/29，2025/10/24，2025/11/14，2025/12/17，2026/03/25</t>
+          <t>2025/03/21，2025/04/28，2025/05/13，2025/06/07，2025/06/21，2025/08/28，2025/09/29，2025/10/24，2025/11/14，2025/12/17，2026/03/25，2026/08/07</t>
         </is>
       </c>
       <c r="F182" t="inlineStr"/>
@@ -7838,7 +7838,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -7907,7 +7907,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/02，2025/12/05，2025/12/30，2026/01/23，2026/01/29，2026/02/23，2026/03/17，2026/03/22，2026/04/19，2026/05/10，2026/06/12，2026/07/22</t>
+          <t>2025/03/22，2025/04/05，2025/04/17，2025/04/21，2025/04/22，2025/04/25，2025/05/08，2025/05/15，2025/05/25，2025/05/29，2025/06/03，2025/06/13，2025/06/23，2025/07/06，2025/07/15，2025/08/03，2025/08/16，2025/09/03，2025/09/10，2025/09/30，2025/10/16，2025/10/22，2025/10/30，2025/11/18，2025/12/02，2025/12/05，2025/12/30，2026/01/23，2026/01/29，2026/02/23，2026/03/17，2026/03/22，2026/04/19，2026/05/10，2026/06/12，2026/07/22，2026/08/08</t>
         </is>
       </c>
       <c r="F184" t="inlineStr"/>
@@ -7918,7 +7918,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>37</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28</t>
+          <t>2025/03/24，2025/04/06，2025/04/15，2025/04/27，2025/05/05，2025/05/22，2025/05/30，2025/06/02，2025/06/06，2025/06/09，2025/06/21，2025/06/27，2025/08/25，2025/09/06，2025/09/10，2025/09/19，2025/10/05，2025/11/21，2025/12/07，2026/01/17，2026/02/14，2026/04/09，2026/05/20，2026/06/19，2026/06/28，2026/07/31</t>
         </is>
       </c>
       <c r="F194" t="inlineStr"/>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -8427,7 +8427,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/09，2026/01/01，2026/02/07，2026/03/25，2026/04/26，2026/06/23</t>
+          <t>2025/03/25，2025/04/11，2025/04/20，2025/05/17，2025/05/22，2025/06/07，2025/06/21，2025/07/06，2025/07/28，2025/09/03，2025/09/14，2025/11/09，2026/01/01，2026/02/07，2026/03/25，2026/04/26，2026/06/23，2026/07/31，2026/07/31</t>
         </is>
       </c>
       <c r="F197" t="inlineStr"/>
@@ -8438,7 +8438,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/28，2025/04/29，2025/05/12，2025/06/06，2025/06/16，2025/07/24，2025/08/01，2025/09/05，2025/09/26，2025/10/28，2025/12/05，2026/01/09，2026/02/19，2026/03/22，2026/04/16</t>
+          <t>2025/03/27，2025/04/03，2025/04/15，2025/04/28，2025/04/29，2025/05/12，2025/06/06，2025/06/16，2025/07/24，2025/08/01，2025/09/05，2025/09/26，2025/10/28，2025/12/05，2026/01/09，2026/02/19，2026/03/22，2026/04/16，2026/08/08</t>
         </is>
       </c>
       <c r="F210" t="inlineStr"/>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -9195,7 +9195,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/01/16，2026/02/02，2026/02/07，2026/03/31，2026/04/17，2026/04/29，2026/05/15，2026/05/19，2026/06/12</t>
+          <t>2025/03/27，2025/05/06，2025/05/16，2025/06/10，2025/07/03，2025/07/13，2025/08/22，2025/10/05，2025/10/23，2025/11/10，2026/01/16，2026/02/02，2026/02/07，2026/03/31，2026/04/17，2026/04/29，2026/05/15，2026/05/19，2026/06/12，2026/08/07</t>
         </is>
       </c>
       <c r="F216" t="inlineStr"/>
@@ -9206,7 +9206,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -9275,7 +9275,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09</t>
+          <t>2025/03/28，2025/07/25，2025/07/26，2025/08/16，2025/09/05，2025/09/29，2025/10/31，2025/12/24，2026/01/16，2026/06/06，2026/07/09，2026/08/08</t>
         </is>
       </c>
       <c r="F218" t="inlineStr"/>
@@ -9286,7 +9286,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -9475,7 +9475,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15</t>
+          <t>2025/03/28，2025/06/07，2025/06/13，2025/06/23，2025/07/20，2025/10/24，2025/11/09，2026/01/09，2026/02/19，2026/05/10，2026/07/10，2026/07/15，2026/07/31</t>
         </is>
       </c>
       <c r="F223" t="inlineStr"/>
@@ -9486,7 +9486,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -9631,7 +9631,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/03，2025/05/26，2025/11/09，2026/05/06，2026/06/10</t>
+          <t>2025/03/28，2025/05/03，2025/05/26，2025/11/09，2026/05/06，2026/06/10，2026/08/02</t>
         </is>
       </c>
       <c r="F227" t="inlineStr"/>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -9671,7 +9671,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20</t>
+          <t>2025/03/28，2025/04/04，2025/04/22，2025/04/29，2025/05/10，2025/05/18，2025/06/02，2025/07/10，2025/08/19，2025/09/10，2025/09/15，2025/10/07，2025/10/26，2025/10/30，2025/11/07，2025/11/24，2025/12/05，2026/01/23，2026/03/09，2026/03/25，2026/06/20，2026/8/16</t>
         </is>
       </c>
       <c r="F228" t="inlineStr"/>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/05/09，2025/06/07，2025/07/31，2025/08/13，2025/08/21，2025/12/16，2026/01/19，2026/05/04</t>
+          <t>2025/03/28，2025/05/09，2025/06/07，2025/07/31，2025/08/13，2025/08/21，2025/12/16，2026/01/19，2026/05/04，2026/07/31</t>
         </is>
       </c>
       <c r="F229" t="inlineStr"/>
@@ -9722,7 +9722,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -9751,7 +9751,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>2025/03/28，2025/04/24，2025/06/02，2025/06/27，2025/09/21，2025/10/07，2025/11/13，2025/12/02</t>
+          <t>2025/03/28，2025/04/24，2025/06/02，2025/06/27，2025/09/21，2025/10/07，2025/11/13，2025/12/02，2026/08/01</t>
         </is>
       </c>
       <c r="F230" t="inlineStr"/>
@@ -9762,7 +9762,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10</t>
+          <t>2025/03/29，2025/04/18，2025/04/24，2025/05/27，2025/06/20，2025/07/03，2025/07/18，2025/08/02，2025/08/24，2025/10/03，2025/10/25，2025/10/28，2025/11/03，2025/11/09，2025/12/23，2026/04/08，2026/04/24，2026/05/21，2026/06/10，2026/08/02</t>
         </is>
       </c>
       <c r="F235" t="inlineStr"/>
@@ -9966,7 +9966,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -9995,7 +9995,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23</t>
+          <t>2025/03/29，2025/04/05，2025/05/30，2025/06/28，2025/09/17，2025/09/18，2025/11/07，2025/11/13，2025/12/02，2026/01/14，2026/01/24，2026/03/07，2026/03/15，2026/04/24，2026/06/06，2026/06/23，2026/08/05，2026/08/05</t>
         </is>
       </c>
       <c r="F236" t="inlineStr"/>
@@ -10006,7 +10006,7 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
@@ -10123,7 +10123,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>2025/03/29，2025/08/12，2025/10/20，2025/11/14，2025/12/02，2026/01/10，2026/02/09，2026/04/18，2026/06/20</t>
+          <t>2025/03/29，2025/08/12，2025/10/20，2025/11/14，2025/12/02，2026/01/10，2026/02/09，2026/04/18，2026/06/20，2026/08/02</t>
         </is>
       </c>
       <c r="F239" t="inlineStr"/>
@@ -10134,7 +10134,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -10163,7 +10163,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/07/13，2025/10/20</t>
+          <t>2025/03/30，2025/07/13，2025/10/20，2026/8/16</t>
         </is>
       </c>
       <c r="F240" t="inlineStr"/>
@@ -10174,7 +10174,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -10403,7 +10403,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18，2026/04/22</t>
+          <t>2025/03/30，2025/04/27，2025/05/19，2025/05/31，2025/08/30，2025/09/02，2025/11/18，2026/04/22，2026/07/31</t>
         </is>
       </c>
       <c r="F246" t="inlineStr"/>
@@ -10414,7 +10414,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/02，2026/04/08，2026/05/01，2026/06/10，2026/06/20</t>
+          <t>2025/04/01，2025/04/17，2025/05/25，2025/07/17，2025/07/21，2025/09/14，2025/10/11，2025/12/02，2026/04/08，2026/05/01，2026/06/10，2026/06/20，2026/08/02</t>
         </is>
       </c>
       <c r="F257" t="inlineStr"/>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>2025/04/02，2025/05/13，2025/05/29，2025/09/04，2025/09/21，2025/10/22，2026/01/01，2026/01/15，2026/05/05</t>
+          <t>2025/04/02，2025/05/13，2025/05/29，2025/09/04，2025/09/21，2025/10/22，2026/01/01，2026/01/15，2026/05/05，2026/8/16</t>
         </is>
       </c>
       <c r="F267" t="inlineStr"/>
@@ -11250,7 +11250,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -11479,7 +11479,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22</t>
+          <t>2025/04/03，2025/04/19，2025/06/16，2025/07/13，2025/07/18，2025/09/19，2025/10/01，2026/01/25，2026/02/14，2026/04/09，2026/06/20，2026/07/22，2026/08/08</t>
         </is>
       </c>
       <c r="F273" t="inlineStr"/>
@@ -11490,7 +11490,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -11723,7 +11723,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>2025/04/03，2025/04/27</t>
+          <t>2025/04/03，2025/04/27，2026/8/16</t>
         </is>
       </c>
       <c r="F279" t="inlineStr"/>
@@ -11734,7 +11734,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28</t>
+          <t>2025/04/04，2025/07/13，2025/07/18，2025/11/03，2025/11/28，2026/8/16</t>
         </is>
       </c>
       <c r="F291" t="inlineStr"/>
@@ -12206,7 +12206,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -12529,7 +12529,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I299" t="inlineStr"/>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>BV1pmh8zDEsy</t>
+        </is>
+      </c>
       <c r="J299" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -12595,7 +12599,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>2025/04/06，2025/04/19，2025/05/03，2025/08/01，2025/10/31，2025/12/15，2026/02/22，2026/02/23，2026/04/17</t>
+          <t>2025/04/06，2025/04/19，2025/05/03，2025/08/01，2025/10/31，2025/12/15，2026/02/22，2026/02/23，2026/04/17，2026/07/31</t>
         </is>
       </c>
       <c r="F301" t="inlineStr"/>
@@ -12606,7 +12610,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -12795,7 +12799,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/05/19，2025/10/01，2025/10/31，2026/01/05，2026/03/25，2026/03/25</t>
+          <t>2025/04/07，2025/05/19，2025/10/01，2025/10/31，2026/01/05，2026/03/25，2026/03/25，2026/08/02</t>
         </is>
       </c>
       <c r="F306" t="inlineStr"/>
@@ -12806,7 +12810,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -12835,7 +12839,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20</t>
+          <t>2025/04/07，2025/04/17，2025/04/19，2025/04/27，2025/04/29，2025/05/20，2025/06/14，2025/07/23，2025/08/29，2025/10/01，2025/11/18，2026/01/03，2026/01/22，2026/02/14，2026/05/20，2026/08/08</t>
         </is>
       </c>
       <c r="F307" t="inlineStr"/>
@@ -12846,7 +12850,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -12915,7 +12919,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20</t>
+          <t>2025/04/08，2025/04/21，2025/04/26，2025/05/10，2025/05/13，2025/05/19，2025/05/30，2025/06/05，2025/06/13，2025/07/05，2025/07/08，2025/07/13，2025/07/15，2025/08/30，2025/09/11，2025/09/18，2025/09/24，2025/09/30，2025/10/30，2025/11/03，2025/11/09，2025/11/26，2025/12/09，2026/01/23，2026/03/13，2026/03/25，2026/04/08，2026/05/23，2026/06/20，2026/08/02</t>
         </is>
       </c>
       <c r="F309" t="inlineStr"/>
@@ -12926,7 +12930,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -13009,7 +13013,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I311" t="inlineStr"/>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>BV1KmdUYhEJu</t>
+        </is>
+      </c>
       <c r="J311" t="inlineStr"/>
     </row>
     <row r="312">
@@ -13031,7 +13039,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/02/23，2026/03/06，2026/04/22，2026/06/10</t>
+          <t>2025/04/08，2025/05/12，2025/08/22，2025/10/01，2025/10/17，2026/02/23，2026/03/06，2026/04/22，2026/06/10，2026/08/05</t>
         </is>
       </c>
       <c r="F312" t="inlineStr"/>
@@ -13042,7 +13050,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -13071,7 +13079,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/09，2025/12/05，2025/12/19，2025/12/26，2026/01/10，2026/01/19，2026/02/10，2026/03/24，2026/04/18，2026/06/06</t>
+          <t>2025/04/08，2025/04/13，2025/04/22，2025/05/01，2025/05/22，2025/06/08，2025/06/29，2025/08/30，2025/09/15，2025/10/10，2025/11/09，2025/12/05，2025/12/19，2025/12/26，2026/01/10，2026/01/19，2026/02/10，2026/03/24，2026/04/18，2026/06/06，2026/08/07</t>
         </is>
       </c>
       <c r="F313" t="inlineStr"/>
@@ -13082,7 +13090,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -13125,7 +13133,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I314" t="inlineStr"/>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>BV1Wvd4YFEz4</t>
+        </is>
+      </c>
       <c r="J314" t="inlineStr"/>
     </row>
     <row r="315">
@@ -13357,7 +13369,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I320" t="inlineStr"/>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>BV1JDoNYYE5V</t>
+        </is>
+      </c>
       <c r="J320" t="inlineStr">
         <is>
           <t>动漫</t>
@@ -13459,7 +13475,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/01/29，2026/02/10，2026/03/09，2026/03/24，2026/04/19，2026/05/21，2026/06/15</t>
+          <t>2025/04/11，2025/05/25，2025/05/29，2025/06/28，2025/07/03，2025/08/13，2025/08/25，2025/09/12，2025/09/11，2025/09/28，2025/10/11，2025/10/30，2025/11/21，2026/01/29，2026/02/10，2026/03/09，2026/03/24，2026/04/19，2026/05/21，2026/06/15，2026/08/02</t>
         </is>
       </c>
       <c r="F323" t="inlineStr"/>
@@ -13470,7 +13486,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -13513,7 +13529,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I324" t="inlineStr"/>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>BV1YmGizgEFL</t>
+        </is>
+      </c>
       <c r="J324" t="inlineStr"/>
     </row>
     <row r="325">
@@ -13585,7 +13605,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I326" t="inlineStr"/>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>BV1MeGdzDEbU</t>
+        </is>
+      </c>
       <c r="J326" t="inlineStr"/>
     </row>
     <row r="327">
@@ -13701,7 +13725,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I329" t="inlineStr"/>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>BV1V1GizrEjQ</t>
+        </is>
+      </c>
       <c r="J329" t="inlineStr"/>
     </row>
     <row r="330">
@@ -14219,7 +14247,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>2025/04/14，2025/10/31</t>
+          <t>2025/04/14，2025/10/31，2026/08/11</t>
         </is>
       </c>
       <c r="F342" t="inlineStr"/>
@@ -14230,7 +14258,7 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
@@ -14827,7 +14855,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/02/18，2026/05/20，2026/07/05</t>
+          <t>2025/04/17，2025/04/29，2025/05/22，2025/05/25，2025/05/31，2025/08/29，2025/09/20，2025/10/09，2025/10/30，2025/12/11，2026/02/18，2026/05/20，2026/07/05，2026/07/31</t>
         </is>
       </c>
       <c r="F357" t="inlineStr"/>
@@ -14838,7 +14866,7 @@
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -14921,7 +14949,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I359" t="inlineStr"/>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>BV1KWVyzXEEL</t>
+        </is>
+      </c>
       <c r="J359" t="inlineStr"/>
     </row>
     <row r="360">
@@ -15139,7 +15171,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>2025/04/18，2025/05/18，2025/06/19，2025/07/15，2025/08/01，2025/09/17，2025/10/28，2025/11/13，2025/11/14，2026/02/10，2026/02/27</t>
+          <t>2025/04/18，2025/05/18，2025/06/19，2025/07/15，2025/08/01，2025/09/17，2025/10/28，2025/11/13，2025/11/14，2026/02/10，2026/02/27，2026/08/02</t>
         </is>
       </c>
       <c r="F365" t="inlineStr"/>
@@ -15150,7 +15182,7 @@
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I365" t="inlineStr">
@@ -15223,7 +15255,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/01/10，2026/03/22，2026/04/24，2026/05/25</t>
+          <t>2025/04/19，2025/07/14，2025/09/12，2025/10/03，2025/10/30，2026/01/10，2026/03/22，2026/04/24，2026/05/25，2026/08/11</t>
         </is>
       </c>
       <c r="F367" t="inlineStr"/>
@@ -15234,7 +15266,7 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
@@ -15343,7 +15375,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>2025/04/19，2025/05/30，2025/07/23，2025/08/23，2025/09/11，2025/12/02，2026/01/26，2026/06/28</t>
+          <t>2025/04/19，2025/05/30，2025/07/23，2025/08/23，2025/09/11，2025/12/02，2026/01/26，2026/06/28，2026/08/07</t>
         </is>
       </c>
       <c r="F370" t="inlineStr"/>
@@ -15354,7 +15386,7 @@
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I370" t="inlineStr">
@@ -15671,7 +15703,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>2025/04/22，2025/04/29，2025/05/03，2025/05/03，2025/06/03，2025/09/02，2025/10/10，2025/10/20，2025/10/31，2026/02/07，2026/03/13</t>
+          <t>2025/04/22，2025/04/29，2025/05/03，2025/05/03，2025/06/03，2025/09/02，2025/10/10，2025/10/20，2025/10/31，2026/02/07，2026/03/13，2026/08/11</t>
         </is>
       </c>
       <c r="F378" t="inlineStr"/>
@@ -15682,7 +15714,7 @@
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I378" t="inlineStr">
@@ -16323,7 +16355,7 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/03，2025/12/30，2026/01/09，2026/04/01，2026/05/23</t>
+          <t>2025/04/25，2025/06/19，2025/06/23，2025/08/12，2025/10/09，2025/11/03，2025/12/30，2026/01/09，2026/04/01，2026/05/23，2026/07/31</t>
         </is>
       </c>
       <c r="F395" t="inlineStr"/>
@@ -16334,7 +16366,7 @@
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I395" t="inlineStr">
@@ -16617,7 +16649,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I402" t="inlineStr"/>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>BV15Bu3zbEcP</t>
+        </is>
+      </c>
       <c r="J402" t="inlineStr"/>
     </row>
     <row r="403">
@@ -16803,7 +16839,7 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>2025/04/28，2025/11/18，2026/02/14，2026/04/09，2026/05/16，2026/06/14</t>
+          <t>2025/04/28，2025/11/18，2026/02/14，2026/04/09，2026/05/16，2026/06/14，2026/08/02</t>
         </is>
       </c>
       <c r="F407" t="inlineStr"/>
@@ -16814,7 +16850,7 @@
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
@@ -16933,7 +16969,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I410" t="inlineStr"/>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>BV1P8GSzFEa7</t>
+        </is>
+      </c>
       <c r="J410" t="inlineStr"/>
     </row>
     <row r="411">
@@ -17009,7 +17049,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I412" t="inlineStr"/>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>BV12dEjz9Etf</t>
+        </is>
+      </c>
       <c r="J412" t="inlineStr"/>
     </row>
     <row r="413">
@@ -17125,7 +17169,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I415" t="inlineStr"/>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>BV116Gdz2ELk</t>
+        </is>
+      </c>
       <c r="J415" t="inlineStr"/>
     </row>
     <row r="416">
@@ -17147,7 +17195,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>2025/05/03，2025/08/28，2025/09/11，2025/10/20，2025/12/09</t>
+          <t>2025/05/03，2025/08/28，2025/09/11，2025/10/20，2025/12/09，2026/8/16</t>
         </is>
       </c>
       <c r="F416" t="inlineStr"/>
@@ -17158,7 +17206,7 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
@@ -17601,7 +17649,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I427" t="inlineStr"/>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>BV1ps55zYEGz</t>
+        </is>
+      </c>
       <c r="J427" t="inlineStr"/>
     </row>
     <row r="428">
@@ -17779,7 +17831,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29</t>
+          <t>2025/05/10，2025/06/10，2025/08/03，2025/09/05，2026/04/29，2026/08/07</t>
         </is>
       </c>
       <c r="F432" t="inlineStr"/>
@@ -17790,7 +17842,7 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
@@ -18139,7 +18191,7 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/01/01，2026/02/10，2026/02/22，2026/03/12，2026/04/05，2026/05/03，2026/05/24，2026/07/03</t>
+          <t>2025/05/17，2025/05/31，2025/06/15，2025/07/23，2025/09/11，2026/01/01，2026/02/10，2026/02/22，2026/03/12，2026/04/05，2026/05/03，2026/05/24，2026/07/03，2026/08/07</t>
         </is>
       </c>
       <c r="F441" t="inlineStr"/>
@@ -18150,7 +18202,7 @@
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
@@ -18233,7 +18285,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I443" t="inlineStr"/>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>BV1tMNXzxEwY</t>
+        </is>
+      </c>
       <c r="J443" t="inlineStr"/>
     </row>
     <row r="444">
@@ -18375,7 +18431,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09</t>
+          <t>2025/05/18，2025/06/07，2025/06/10，2025/06/12，2025/06/13，2025/06/17，2025/06/23，2025/07/08，2025/07/13，2025/07/20，2025/07/31，2025/09/17，2025/09/26，2025/10/07，2025/11/13，2025/12/17，2026/01/02，2026/03/17，2026/04/29，2026/05/10，2026/07/09，2026/07/31，2026/08/11</t>
         </is>
       </c>
       <c r="F447" t="inlineStr"/>
@@ -18386,7 +18442,7 @@
       </c>
       <c r="H447" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I447" t="inlineStr">
@@ -18455,7 +18511,7 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/12/16，2025/12/24</t>
+          <t>2025/05/19，2025/12/16，2025/12/24，2026/8/16</t>
         </is>
       </c>
       <c r="F449" t="inlineStr"/>
@@ -18466,7 +18522,7 @@
       </c>
       <c r="H449" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I449" t="inlineStr">
@@ -18495,7 +18551,7 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/07/13，2025/08/21，2025/12/17，2026/05/23</t>
+          <t>2025/05/19，2025/07/13，2025/08/21，2025/12/17，2026/05/23，2026/08/11</t>
         </is>
       </c>
       <c r="F450" t="inlineStr"/>
@@ -18506,7 +18562,7 @@
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I450" t="inlineStr">
@@ -18549,7 +18605,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I451" t="inlineStr"/>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>BV1EdEQzrEyw</t>
+        </is>
+      </c>
       <c r="J451" t="inlineStr"/>
     </row>
     <row r="452">
@@ -18575,7 +18635,7 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>2025/05/19，2025/07/13，2025/10/30，2025/10/31，2025/12/24，2026/01/09，2026/04/09，2026/05/07</t>
+          <t>2025/05/19，2025/07/13，2025/10/30，2025/10/31，2025/12/24，2026/01/09，2026/04/09，2026/05/07，2026/07/31</t>
         </is>
       </c>
       <c r="F452" t="inlineStr"/>
@@ -18586,7 +18646,7 @@
       </c>
       <c r="H452" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I452" t="inlineStr">
@@ -18615,7 +18675,7 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/06，2026/03/22，2026/05/01</t>
+          <t>2025/05/22，2025/05/31，2025/06/07，2025/06/10，2025/08/02，2025/10/07，2025/12/06，2026/03/22，2026/05/01，2026/8/16</t>
         </is>
       </c>
       <c r="F453" t="inlineStr"/>
@@ -18626,7 +18686,7 @@
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I453" t="inlineStr">
@@ -18819,7 +18879,7 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>2025/05/22</t>
+          <t>2025/05/22，2026/07/30</t>
         </is>
       </c>
       <c r="F458" t="inlineStr"/>
@@ -18830,7 +18890,7 @@
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I458" t="inlineStr">
@@ -18863,7 +18923,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/01/05，2026/02/02，2026/03/17，2026/05/10，2026/06/14，2026/06/15</t>
+          <t>2025/05/22，2025/05/25，2025/05/31，2025/06/03，2025/06/10，2025/06/13，2025/06/23，2025/07/23，2025/07/24，2025/07/27，2025/08/22，2025/09/06，2025/10/28，2025/10/30，2025/11/10，2025/11/19，2026/01/05，2026/02/02，2026/03/17，2026/05/10，2026/06/14，2026/06/15，2026/07/31</t>
         </is>
       </c>
       <c r="F459" t="inlineStr"/>
@@ -18874,7 +18934,7 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
@@ -19041,7 +19101,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I463" t="inlineStr"/>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>BV1ihjpzEEWS</t>
+        </is>
+      </c>
       <c r="J463" t="inlineStr"/>
     </row>
     <row r="464">
@@ -19077,7 +19141,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I464" t="inlineStr"/>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>BV1ofuNzSEmK</t>
+        </is>
+      </c>
       <c r="J464" t="inlineStr"/>
     </row>
     <row r="465">
@@ -19179,7 +19247,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/01/28，2026/04/08</t>
+          <t>2025/05/24，2025/07/13，2025/08/23，2025/09/29，2025/12/24，2025/12/30，2026/01/28，2026/04/08，2026/8/16</t>
         </is>
       </c>
       <c r="F467" t="inlineStr"/>
@@ -19190,7 +19258,7 @@
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
@@ -19313,7 +19381,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I470" t="inlineStr"/>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>BV1CZj3zcEhL</t>
+        </is>
+      </c>
       <c r="J470" t="inlineStr"/>
     </row>
     <row r="471">
@@ -19349,7 +19421,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I471" t="inlineStr"/>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>BV1nF33zGE8P</t>
+        </is>
+      </c>
       <c r="J471" t="inlineStr"/>
     </row>
     <row r="472">
@@ -19465,7 +19541,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I474" t="inlineStr"/>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>BV1CN7pzFEVF</t>
+        </is>
+      </c>
       <c r="J474" t="inlineStr"/>
     </row>
     <row r="475">
@@ -19487,7 +19567,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/08/23，2025/10/11</t>
+          <t>2025/05/30，2025/08/23，2025/10/11，2026/8/16</t>
         </is>
       </c>
       <c r="F475" t="inlineStr"/>
@@ -19498,7 +19578,7 @@
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I475" t="inlineStr">
@@ -19541,7 +19621,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I476" t="inlineStr"/>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>BV1MF7PzDESp</t>
+        </is>
+      </c>
       <c r="J476" t="inlineStr"/>
     </row>
     <row r="477">
@@ -19563,7 +19647,7 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/07/13，2025/10/31，2026/03/05</t>
+          <t>2025/05/30，2025/07/13，2025/10/31，2026/03/05，2026/08/08</t>
         </is>
       </c>
       <c r="F477" t="inlineStr"/>
@@ -19574,7 +19658,7 @@
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I477" t="inlineStr">
@@ -19683,7 +19767,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>2025/05/30，2025/05/31，2025/05/31，2025/06/02，2025/06/03，2025/06/05，2025/06/19，2025/06/26，2025/07/03，2025/07/14，2025/08/02，2025/08/24，2025/09/03，2025/09/18，2025/10/07，2025/11/19，2025/12/11，2026/01/10，2026/01/22，2026/03/25，2026/06/28</t>
+          <t>2025/05/30，2025/05/31，2025/05/31，2025/06/02，2025/06/03，2025/06/05，2025/06/19，2025/06/26，2025/07/03，2025/07/14，2025/08/02，2025/08/24，2025/09/03，2025/09/18，2025/10/07，2025/11/19，2025/12/11，2026/01/10，2026/01/22，2026/03/25，2026/06/28，2026/08/03</t>
         </is>
       </c>
       <c r="F480" t="inlineStr"/>
@@ -19694,7 +19778,7 @@
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I480" t="inlineStr">
@@ -19723,7 +19807,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>2025/05/31，2025/06/02，2025/06/23，2025/09/15，2025/09/27，2025/10/17</t>
+          <t>2025/05/31，2025/06/02，2025/06/23，2025/09/15，2025/09/27，2025/10/17，2026/8/16</t>
         </is>
       </c>
       <c r="F481" t="inlineStr"/>
@@ -19734,7 +19818,7 @@
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I481" t="inlineStr">
@@ -19777,7 +19861,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I482" t="inlineStr"/>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>BV1Ey7NzzEcC</t>
+        </is>
+      </c>
       <c r="J482" t="inlineStr"/>
     </row>
     <row r="483">
@@ -19813,7 +19901,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I483" t="inlineStr"/>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>BV1qm7NzqEAT</t>
+        </is>
+      </c>
       <c r="J483" t="inlineStr"/>
     </row>
     <row r="484">
@@ -19853,7 +19945,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I484" t="inlineStr"/>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>BV16WypB3EX6</t>
+        </is>
+      </c>
       <c r="J484" t="inlineStr"/>
     </row>
     <row r="485">
@@ -20101,7 +20197,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I490" t="inlineStr"/>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>BV1ny7rzLE4i</t>
+        </is>
+      </c>
       <c r="J490" t="inlineStr"/>
     </row>
     <row r="491">
@@ -20285,7 +20385,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I495" t="inlineStr"/>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>BV1r37mzwE3A</t>
+        </is>
+      </c>
       <c r="J495" t="inlineStr"/>
     </row>
     <row r="496">
@@ -20401,7 +20505,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I498" t="inlineStr"/>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>BV1YY7SzREB6</t>
+        </is>
+      </c>
       <c r="J498" t="inlineStr"/>
     </row>
     <row r="499">
@@ -20437,7 +20545,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I499" t="inlineStr"/>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>BV1zp7SzaEq7</t>
+        </is>
+      </c>
       <c r="J499" t="inlineStr"/>
     </row>
     <row r="500">
@@ -20473,7 +20585,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I500" t="inlineStr"/>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>BV1jV7XzKEk1</t>
+        </is>
+      </c>
       <c r="J500" t="inlineStr"/>
     </row>
     <row r="501">
@@ -20589,7 +20705,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I503" t="inlineStr"/>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>BV16xwozUELq</t>
+        </is>
+      </c>
       <c r="J503" t="inlineStr"/>
     </row>
     <row r="504">
@@ -20701,7 +20821,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I506" t="inlineStr"/>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>BV15gTjzKEAJ</t>
+        </is>
+      </c>
       <c r="J506" t="inlineStr"/>
     </row>
     <row r="507">
@@ -20737,7 +20861,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I507" t="inlineStr"/>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>BV1FaT2zYEEQ</t>
+        </is>
+      </c>
       <c r="J507" t="inlineStr"/>
     </row>
     <row r="508">
@@ -20773,7 +20901,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I508" t="inlineStr"/>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>BV1joT1z4E8u</t>
+        </is>
+      </c>
       <c r="J508" t="inlineStr"/>
     </row>
     <row r="509">
@@ -20875,7 +21007,7 @@
       </c>
       <c r="E511" t="inlineStr">
         <is>
-          <t>2025/06/09，2025/09/26，2025/10/17，2025/10/25，2026/05/01</t>
+          <t>2025/06/09，2025/09/26，2025/10/17，2025/10/25，2026/05/01，2026/08/02</t>
         </is>
       </c>
       <c r="F511" t="inlineStr"/>
@@ -20886,7 +21018,7 @@
       </c>
       <c r="H511" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I511" t="inlineStr">
@@ -21159,7 +21291,7 @@
       </c>
       <c r="E518" t="inlineStr">
         <is>
-          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/02，2025/12/09，2025/12/16，2025/12/26，2026/01/05，2026/01/15，2026/01/28，2026/03/06，2026/04/22，2026/05/10，2026/05/15，2026/06/19，2026/07/09</t>
+          <t>2025/06/15，2025/06/15，2025/06/16，2025/06/17，2025/06/19，2025/06/27，2025/07/03，2025/07/05，2025/07/11，2025/07/25，2025/08/01，2025/08/03，2025/08/13，2025/09/03，2025/09/12，2025/09/24，2025/10/07，2025/10/24，2025/11/13，2025/12/02，2025/12/09，2025/12/16，2025/12/26，2026/01/05，2026/01/15，2026/01/28，2026/03/06，2026/04/22，2026/05/10，2026/05/15，2026/06/19，2026/07/09，2026/07/31</t>
         </is>
       </c>
       <c r="F518" t="inlineStr"/>
@@ -21170,7 +21302,7 @@
       </c>
       <c r="H518" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="I518" t="inlineStr">
@@ -21213,7 +21345,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I519" t="inlineStr"/>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>BV11DNtzSEY2</t>
+        </is>
+      </c>
       <c r="J519" t="inlineStr"/>
     </row>
     <row r="520">
@@ -21369,7 +21505,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I523" t="inlineStr"/>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>BV1K1N5z2EHA</t>
+        </is>
+      </c>
       <c r="J523" t="inlineStr"/>
     </row>
     <row r="524">
@@ -21605,7 +21745,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I529" t="inlineStr"/>
+      <c r="I529" t="inlineStr">
+        <is>
+          <t>BV1tH3FztEpR</t>
+        </is>
+      </c>
       <c r="J529" t="inlineStr"/>
     </row>
     <row r="530">
@@ -21627,7 +21771,7 @@
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/07，2025/11/21，2025/12/02，2025/12/17，2026/01/01，2026/01/05，2026/01/14，2026/01/22，2026/01/24，2026/02/02，2026/03/05，2026/03/15，2026/04/01，2026/05/04，2026/05/25，2026/06/20，2026/07/05，2026/07/18，2026/07/28</t>
+          <t>2025/06/19，2025/07/14，2025/07/17，2025/07/28，2025/08/03，2025/08/08，2025/08/22，2025/09/17，2025/09/26，2025/09/30，2025/10/12，2025/10/16，2025/11/07，2025/11/21，2025/12/02，2025/12/17，2026/01/01，2026/01/05，2026/01/14，2026/01/22，2026/01/24，2026/02/02，2026/03/05，2026/03/15，2026/04/01，2026/05/04，2026/05/25，2026/06/20，2026/07/05，2026/07/18，2026/07/28，2026/08/11</t>
         </is>
       </c>
       <c r="F530" t="inlineStr"/>
@@ -21638,7 +21782,7 @@
       </c>
       <c r="H530" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="I530" t="inlineStr">
@@ -21831,7 +21975,7 @@
       </c>
       <c r="E535" t="inlineStr">
         <is>
-          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/02/18，2026/03/09，2026/04/16，2026/04/24，2026/05/15，2026/05/23，2026/06/12，2026/07/22</t>
+          <t>2025/06/20，2025/06/21，2025/07/08，2025/07/13，2025/07/18，2025/07/28，2025/08/01，2025/08/03，2025/08/04，2025/08/16，2025/09/03，2025/09/13，2025/09/19，2025/10/23，2025/10/28，2025/11/10，2025/11/13，2025/11/18，2025/12/11，2025/12/16，2026/02/18，2026/03/09，2026/04/16，2026/04/24，2026/05/15，2026/05/23，2026/06/12，2026/07/22，2026/08/11</t>
         </is>
       </c>
       <c r="F535" t="inlineStr"/>
@@ -21842,7 +21986,7 @@
       </c>
       <c r="H535" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="I535" t="inlineStr">
@@ -21925,7 +22069,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I537" t="inlineStr"/>
+      <c r="I537" t="inlineStr">
+        <is>
+          <t>BV1BCMp6DEtt</t>
+        </is>
+      </c>
       <c r="J537" t="inlineStr"/>
     </row>
     <row r="538">
@@ -21961,7 +22109,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I538" t="inlineStr"/>
+      <c r="I538" t="inlineStr">
+        <is>
+          <t>BV1ZFKhzLEqz</t>
+        </is>
+      </c>
       <c r="J538" t="inlineStr"/>
     </row>
     <row r="539">
@@ -21997,7 +22149,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I539" t="inlineStr"/>
+      <c r="I539" t="inlineStr">
+        <is>
+          <t>BV1XbK8ziE7s</t>
+        </is>
+      </c>
       <c r="J539" t="inlineStr"/>
     </row>
     <row r="540">
@@ -22019,7 +22175,7 @@
       </c>
       <c r="E540" t="inlineStr">
         <is>
-          <t>2025/06/23，2025/10/19，2026/01/19</t>
+          <t>2025/06/23，2025/10/19，2026/01/19，2026/8/16</t>
         </is>
       </c>
       <c r="F540" t="inlineStr"/>
@@ -22030,7 +22186,7 @@
       </c>
       <c r="H540" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I540" t="inlineStr">
@@ -22189,7 +22345,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I544" t="inlineStr"/>
+      <c r="I544" t="inlineStr">
+        <is>
+          <t>BV178KfzbEJ6</t>
+        </is>
+      </c>
       <c r="J544" t="inlineStr"/>
     </row>
     <row r="545">
@@ -22215,7 +22375,7 @@
       </c>
       <c r="E545" t="inlineStr">
         <is>
-          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/01/14，2026/01/22，2026/02/19，2026/03/13，2026/04/12，2026/05/10，2026/06/17</t>
+          <t>2025/06/26，2025/06/27，2025/07/14，2025/07/17，2025/08/23，2025/09/21，2025/10/28，2025/11/10，2026/01/14，2026/01/22，2026/02/19，2026/03/13，2026/04/12，2026/05/10，2026/06/17，2026/08/08</t>
         </is>
       </c>
       <c r="F545" t="inlineStr"/>
@@ -22226,7 +22386,7 @@
       </c>
       <c r="H545" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I545" t="inlineStr">
@@ -22299,7 +22459,7 @@
       </c>
       <c r="E547" t="inlineStr">
         <is>
-          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/01/24，2026/02/09，2026/03/06，2026/03/22，2026/04/11，2026/04/30，2026/05/26，2026/06/18</t>
+          <t>2025/06/27，2025/09/08，2025/10/13，2025/10/16，2026/01/24，2026/02/09，2026/03/06，2026/03/22，2026/04/11，2026/04/30，2026/05/26，2026/06/18，2026/08/03</t>
         </is>
       </c>
       <c r="F547" t="inlineStr">
@@ -22314,7 +22474,7 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
@@ -22405,7 +22565,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I549" t="inlineStr"/>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>BV17iK6zkEYv</t>
+        </is>
+      </c>
       <c r="J549" t="inlineStr"/>
     </row>
     <row r="550">
@@ -22481,7 +22645,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I551" t="inlineStr"/>
+      <c r="I551" t="inlineStr">
+        <is>
+          <t>BV1Fv3Xz8ETi</t>
+        </is>
+      </c>
       <c r="J551" t="inlineStr"/>
     </row>
     <row r="552">
@@ -22543,7 +22711,7 @@
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26</t>
+          <t>2025/06/29，2025/07/03，2025/07/14，2025/09/17，2025/11/13，2025/11/27，2025/12/16，2026/05/26，2026/8/16</t>
         </is>
       </c>
       <c r="F553" t="inlineStr"/>
@@ -22554,7 +22722,7 @@
       </c>
       <c r="H553" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I553" t="inlineStr">
@@ -22583,7 +22751,7 @@
       </c>
       <c r="E554" t="inlineStr">
         <is>
-          <t>2025/06/29</t>
+          <t>2025/06/29，2026/08/11</t>
         </is>
       </c>
       <c r="F554" t="inlineStr"/>
@@ -22594,10 +22762,14 @@
       </c>
       <c r="H554" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I554" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>BV1KBgCzkELn</t>
+        </is>
+      </c>
       <c r="J554" t="inlineStr"/>
     </row>
     <row r="555">
@@ -22633,7 +22805,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I555" t="inlineStr"/>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>BV158yXBUENQ</t>
+        </is>
+      </c>
       <c r="J555" t="inlineStr"/>
     </row>
     <row r="556">
@@ -22669,7 +22845,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I556" t="inlineStr"/>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>BV1MegCzLEbb</t>
+        </is>
+      </c>
       <c r="J556" t="inlineStr"/>
     </row>
     <row r="557">
@@ -22705,7 +22885,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I557" t="inlineStr"/>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>BV14v3PzNEcG</t>
+        </is>
+      </c>
       <c r="J557" t="inlineStr"/>
     </row>
     <row r="558">
@@ -22741,7 +22925,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I558" t="inlineStr"/>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>BV1pHGFzHEHx</t>
+        </is>
+      </c>
       <c r="J558" t="inlineStr"/>
     </row>
     <row r="559">
@@ -22777,7 +22965,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I559" t="inlineStr"/>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>BV1ergkzDEuP</t>
+        </is>
+      </c>
       <c r="J559" t="inlineStr"/>
     </row>
     <row r="560">
@@ -22889,7 +23081,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I562" t="inlineStr"/>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>BV1G8g1zdELq</t>
+        </is>
+      </c>
       <c r="J562" t="inlineStr"/>
     </row>
     <row r="563">
@@ -22965,7 +23161,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I564" t="inlineStr"/>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>BV1Bm3izjEJZ</t>
+        </is>
+      </c>
       <c r="J564" t="inlineStr"/>
     </row>
     <row r="565">
@@ -23637,7 +23837,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I581" t="inlineStr"/>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>BV1mvM9zqELY</t>
+        </is>
+      </c>
       <c r="J581" t="inlineStr"/>
     </row>
     <row r="582">
@@ -23833,7 +24037,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I586" t="inlineStr"/>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>BV1Jkgtz9ELP</t>
+        </is>
+      </c>
       <c r="J586" t="inlineStr"/>
     </row>
     <row r="587">
@@ -23895,7 +24103,7 @@
       </c>
       <c r="E588" t="inlineStr">
         <is>
-          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/01/09，2026/04/02，2026/04/24，2026/05/22，2026/06/12，2026/06/17</t>
+          <t>2025/07/17，2025/07/18，2025/07/24，2025/07/26，2025/07/31，2025/09/26，2025/09/29，2025/10/09，2025/12/26，2026/01/09，2026/04/02，2026/04/24，2026/05/22，2026/06/12，2026/06/17，2026/08/11</t>
         </is>
       </c>
       <c r="F588" t="inlineStr"/>
@@ -23906,7 +24114,7 @@
       </c>
       <c r="H588" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I588" t="inlineStr">
@@ -24097,7 +24305,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I593" t="inlineStr"/>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>BV15Whuz2E7Y</t>
+        </is>
+      </c>
       <c r="J593" t="inlineStr"/>
     </row>
     <row r="594">
@@ -24133,7 +24345,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I594" t="inlineStr"/>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>BV1ktaZzwEZT</t>
+        </is>
+      </c>
       <c r="J594" t="inlineStr"/>
     </row>
     <row r="595">
@@ -24169,7 +24385,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I595" t="inlineStr"/>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>BV151gWzKEos</t>
+        </is>
+      </c>
       <c r="J595" t="inlineStr"/>
     </row>
     <row r="596">
@@ -24191,7 +24411,7 @@
       </c>
       <c r="E596" t="inlineStr">
         <is>
-          <t>2025/07/23，2025/12/12，2026/02/25，2026/04/09，2026/04/14</t>
+          <t>2025/07/23，2025/12/12，2026/02/25，2026/04/09，2026/04/14，2026/08/02</t>
         </is>
       </c>
       <c r="F596" t="inlineStr"/>
@@ -24202,7 +24422,7 @@
       </c>
       <c r="H596" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I596" t="inlineStr">
@@ -24329,7 +24549,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I599" t="inlineStr"/>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>BV1d68pzEEd3</t>
+        </is>
+      </c>
       <c r="J599" t="inlineStr"/>
     </row>
     <row r="600">
@@ -24485,7 +24709,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I603" t="inlineStr"/>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>BV12o8nzfEPr</t>
+        </is>
+      </c>
       <c r="J603" t="inlineStr"/>
     </row>
     <row r="604">
@@ -24561,7 +24789,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I605" t="inlineStr"/>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>BV1x6pgzLE5J</t>
+        </is>
+      </c>
       <c r="J605" t="inlineStr"/>
     </row>
     <row r="606">
@@ -24775,7 +25007,7 @@
       </c>
       <c r="E611" t="inlineStr">
         <is>
-          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/02，2025/12/17，2026/01/14，2026/02/02，2026/03/22，2026/04/01，2026/04/08，2026/05/15，2026/06/10</t>
+          <t>2025/08/09，2025/08/10，2025/08/13，2025/08/22，2025/08/25，2025/09/03，2025/09/05，2025/09/20，2025/09/29，2025/10/05，2025/10/22，2025/11/14，2025/12/02，2025/12/17，2026/01/14，2026/02/02，2026/03/22，2026/04/01，2026/04/08，2026/05/15，2026/06/10，2026/07/31</t>
         </is>
       </c>
       <c r="F611" t="inlineStr"/>
@@ -24786,7 +25018,7 @@
       </c>
       <c r="H611" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I611" t="inlineStr">
@@ -24804,7 +25036,7 @@
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>原创曲（未命名）</t>
+          <t>优尼瓦思电力</t>
         </is>
       </c>
       <c r="C612" t="inlineStr"/>
@@ -24815,7 +25047,7 @@
       </c>
       <c r="E612" t="inlineStr">
         <is>
-          <t>2025/08/09，2026/03/13，2026/03/27</t>
+          <t>2025/08/09，2026/03/13，2026/03/27，2026/08/02</t>
         </is>
       </c>
       <c r="F612" t="inlineStr">
@@ -24830,7 +25062,7 @@
       </c>
       <c r="H612" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I612" t="inlineStr">
@@ -24895,7 +25127,7 @@
       </c>
       <c r="E614" t="inlineStr">
         <is>
-          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/01，2025/11/26，2025/12/30，2026/01/10，2026/02/18，2026/04/10，2026/04/23，2026/05/23，2026/06/18，2026/07/13</t>
+          <t>2025/08/12，2025/09/05，2025/09/05，2025/09/17，2025/09/24，2025/09/28，2025/10/01，2025/10/10，2025/10/17，2025/10/23，2025/11/01，2025/11/26，2025/12/30，2026/01/10，2026/02/18，2026/04/10，2026/04/23，2026/05/23，2026/06/18，2026/07/13，2026/08/07</t>
         </is>
       </c>
       <c r="F614" t="inlineStr"/>
@@ -24906,7 +25138,7 @@
       </c>
       <c r="H614" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="I614" t="inlineStr">
@@ -24935,7 +25167,7 @@
       </c>
       <c r="E615" t="inlineStr">
         <is>
-          <t>2025/08/21，2026/01/16，2026/02/02，2026/03/17，2026/04/08，2026/06/14</t>
+          <t>2025/08/21，2026/01/16，2026/02/02，2026/03/17，2026/04/08，2026/06/14，2026/08/02</t>
         </is>
       </c>
       <c r="F615" t="inlineStr"/>
@@ -24946,7 +25178,7 @@
       </c>
       <c r="H615" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I615" t="inlineStr">
@@ -25113,7 +25345,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I619" t="inlineStr"/>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>BV11Uerz8E9J</t>
+        </is>
+      </c>
       <c r="J619" t="inlineStr"/>
     </row>
     <row r="620">
@@ -25345,7 +25581,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I625" t="inlineStr"/>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>BV1FQYMz4E82</t>
+        </is>
+      </c>
       <c r="J625" t="inlineStr"/>
     </row>
     <row r="626">
@@ -25581,7 +25821,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I631" t="inlineStr"/>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>BV1WhHrzfEYw</t>
+        </is>
+      </c>
       <c r="J631" t="inlineStr"/>
     </row>
     <row r="632">
@@ -25657,7 +25901,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I633" t="inlineStr"/>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>BV17opgzeE7g</t>
+        </is>
+      </c>
       <c r="J633" t="inlineStr"/>
     </row>
     <row r="634">
@@ -26335,7 +26583,7 @@
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>2025/09/15，2026/03/13</t>
+          <t>2025/09/15，2026/03/13，2026/08/02</t>
         </is>
       </c>
       <c r="F651" t="inlineStr"/>
@@ -26346,7 +26594,7 @@
       </c>
       <c r="H651" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I651" t="inlineStr">
@@ -26647,7 +26895,7 @@
       </c>
       <c r="E659" t="inlineStr">
         <is>
-          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05</t>
+          <t>2025/09/21，2025/09/21，2025/09/22，2025/09/22，2025/09/24，2025/09/27，2025/09/29，2025/10/03，2025/10/05，2025/10/09，2025/10/18，2025/10/22，2025/10/26，2025/11/01，2025/11/09，2025/11/19，2025/11/22，2025/11/28，2025/12/08，2025/12/22，2026/01/05，2026/01/14，2026/01/22，2026/02/07，2026/02/10，2026/03/08，2026/03/22，2026/04/18，2026/05/01，2026/05/20，2026/06/10，2026/06/25，2026/07/05，2026/07/31</t>
         </is>
       </c>
       <c r="F659" t="inlineStr"/>
@@ -26658,7 +26906,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -26741,7 +26989,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I661" t="inlineStr"/>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>BV1VenwzhEE1</t>
+        </is>
+      </c>
       <c r="J661" t="inlineStr"/>
     </row>
     <row r="662">
@@ -26835,7 +27087,7 @@
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>2025/09/22，2025/10/09，2025/12/05</t>
+          <t>2025/09/22，2025/10/09，2025/12/05，2026/8/16</t>
         </is>
       </c>
       <c r="F664" t="inlineStr"/>
@@ -26846,10 +27098,14 @@
       </c>
       <c r="H664" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I664" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>BV1CJnKzxErq</t>
+        </is>
+      </c>
       <c r="J664" t="inlineStr"/>
     </row>
     <row r="665">
@@ -27019,7 +27275,7 @@
       </c>
       <c r="E669" t="inlineStr">
         <is>
-          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16</t>
+          <t>2025/09/24，2025/09/26，2025/09/28，2025/09/29，2025/10/01，2025/10/07，2025/10/10，2025/10/11，2025/10/17，2025/10/23，2025/10/28，2025/12/26，2026/02/05，2026/07/16，2026/07/31</t>
         </is>
       </c>
       <c r="F669" t="inlineStr"/>
@@ -27030,7 +27286,7 @@
       </c>
       <c r="H669" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I669" t="inlineStr">
@@ -27291,7 +27547,7 @@
       </c>
       <c r="E676" t="inlineStr">
         <is>
-          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/02，2025/12/11，2026/01/09，2026/01/14，2026/02/07，2026/03/22，2026/04/27，2026/05/25，2026/06/20，2026/07/09，2026/07/26</t>
+          <t>2025/09/29，2025/09/30，2025/10/05，2025/10/07，2025/10/11，2025/10/16，2025/10/19，2025/10/22，2025/10/25，2025/11/19，2025/12/02，2025/12/11，2026/01/09，2026/01/14，2026/02/07，2026/03/22，2026/04/27，2026/05/25，2026/06/20，2026/07/09，2026/07/26，2026/08/11</t>
         </is>
       </c>
       <c r="F676" t="inlineStr"/>
@@ -27302,7 +27558,7 @@
       </c>
       <c r="H676" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="I676" t="inlineStr">
@@ -27385,7 +27641,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I678" t="inlineStr"/>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>BV1ZHn1ztEyz</t>
+        </is>
+      </c>
       <c r="J678" t="inlineStr"/>
     </row>
     <row r="679">
@@ -27407,7 +27667,7 @@
       </c>
       <c r="E679" t="inlineStr">
         <is>
-          <t>2025/09/30，2025/10/01，2025/10/11，2025/10/17，2025/10/26</t>
+          <t>2025/09/30，2025/10/01，2025/10/11，2025/10/17，2025/10/26，2026/8/16</t>
         </is>
       </c>
       <c r="F679" t="inlineStr"/>
@@ -27418,10 +27678,14 @@
       </c>
       <c r="H679" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="I679" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>BV1tksmz4EF8</t>
+        </is>
+      </c>
       <c r="J679" t="inlineStr"/>
     </row>
     <row r="680">
@@ -27497,7 +27761,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I681" t="inlineStr"/>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>BV15ZHpzbEZN</t>
+        </is>
+      </c>
       <c r="J681" t="inlineStr"/>
     </row>
     <row r="682">
@@ -27533,7 +27801,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I682" t="inlineStr"/>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>BV1vdHpzfEJe</t>
+        </is>
+      </c>
       <c r="J682" t="inlineStr"/>
     </row>
     <row r="683">
@@ -27681,7 +27953,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I686" t="inlineStr"/>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>BV1xPxgzDEAv</t>
+        </is>
+      </c>
       <c r="J686" t="inlineStr"/>
     </row>
     <row r="687">
@@ -27703,7 +27979,7 @@
       </c>
       <c r="E687" t="inlineStr">
         <is>
-          <t>2025/10/07，2025/10/12，2025/10/22，2026/03/24，2026/04/02</t>
+          <t>2025/10/07，2025/10/12，2025/10/22，2026/03/24，2026/04/02，2026/08/07</t>
         </is>
       </c>
       <c r="F687" t="inlineStr"/>
@@ -27714,7 +27990,7 @@
       </c>
       <c r="H687" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I687" t="inlineStr">
@@ -27955,7 +28231,7 @@
       </c>
       <c r="E693" t="inlineStr">
         <is>
-          <t>2025/10/13，2025/10/18，2026/03/15</t>
+          <t>2025/10/13，2025/10/18，2026/03/15，2026/08/09</t>
         </is>
       </c>
       <c r="F693" t="inlineStr"/>
@@ -27966,7 +28242,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">
@@ -28315,7 +28591,7 @@
       </c>
       <c r="E702" t="inlineStr">
         <is>
-          <t>2025/10/23</t>
+          <t>2025/10/23，2026/8/16</t>
         </is>
       </c>
       <c r="F702" t="inlineStr"/>
@@ -28326,10 +28602,14 @@
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I702" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I702" t="inlineStr">
+        <is>
+          <t>BV1gabm6ZEH1</t>
+        </is>
+      </c>
       <c r="J702" t="inlineStr"/>
     </row>
     <row r="703">
@@ -28477,7 +28757,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I706" t="inlineStr"/>
+      <c r="I706" t="inlineStr">
+        <is>
+          <t>BV1DasVzNEqy</t>
+        </is>
+      </c>
       <c r="J706" t="inlineStr"/>
     </row>
     <row r="707">
@@ -28513,7 +28797,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I707" t="inlineStr"/>
+      <c r="I707" t="inlineStr">
+        <is>
+          <t>BV1kUsVzWECP</t>
+        </is>
+      </c>
       <c r="J707" t="inlineStr"/>
     </row>
     <row r="708">
@@ -28549,7 +28837,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I708" t="inlineStr"/>
+      <c r="I708" t="inlineStr">
+        <is>
+          <t>BV1s8sjzPEbJ</t>
+        </is>
+      </c>
       <c r="J708" t="inlineStr"/>
     </row>
     <row r="709">
@@ -28683,7 +28975,7 @@
       </c>
       <c r="E712" t="inlineStr">
         <is>
-          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/01，2025/11/12，2025/11/26，2025/12/08，2026/01/02，2026/01/05，2026/01/09，2026/02/23，2026/03/14，2026/03/29，2026/04/24，2026/07/09</t>
+          <t>2025/10/24，2025/10/25，2025/10/28，2025/11/01，2025/11/12，2025/11/26，2025/12/08，2026/01/02，2026/01/05，2026/01/09，2026/02/23，2026/03/14，2026/03/29，2026/04/24，2026/07/09，2026/08/11</t>
         </is>
       </c>
       <c r="F712" t="inlineStr"/>
@@ -28694,7 +28986,7 @@
       </c>
       <c r="H712" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I712" t="inlineStr">
@@ -28767,7 +29059,7 @@
       </c>
       <c r="E714" t="inlineStr">
         <is>
-          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10</t>
+          <t>2025/10/28，2025/11/01，2025/11/12，2025/12/19，2026/02/08，2026/02/10，2026/05/10，2026/8/16</t>
         </is>
       </c>
       <c r="F714" t="inlineStr"/>
@@ -28778,7 +29070,7 @@
       </c>
       <c r="H714" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I714" t="inlineStr">
@@ -28897,7 +29189,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I717" t="inlineStr"/>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>BV1sDyXBNENn</t>
+        </is>
+      </c>
       <c r="J717" t="inlineStr"/>
     </row>
     <row r="718">
@@ -28919,7 +29215,7 @@
       </c>
       <c r="E718" t="inlineStr">
         <is>
-          <t>2025/11/03，2026/04/24</t>
+          <t>2025/11/03，2026/04/24，2026/08/11</t>
         </is>
       </c>
       <c r="F718" t="inlineStr"/>
@@ -28930,7 +29226,7 @@
       </c>
       <c r="H718" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I718" t="inlineStr">
@@ -29013,7 +29309,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I720" t="inlineStr"/>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>BV1qAkDBrE7e</t>
+        </is>
+      </c>
       <c r="J720" t="inlineStr"/>
     </row>
     <row r="721">
@@ -29259,7 +29559,7 @@
       </c>
       <c r="E727" t="inlineStr">
         <is>
-          <t>2025/11/14</t>
+          <t>2025/11/14，2026/08/02</t>
         </is>
       </c>
       <c r="F727" t="inlineStr"/>
@@ -29270,10 +29570,14 @@
       </c>
       <c r="H727" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I727" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>BV1a23Z6jE7P</t>
+        </is>
+      </c>
       <c r="J727" t="inlineStr"/>
     </row>
     <row r="728">
@@ -29309,7 +29613,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I728" t="inlineStr"/>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>BV1mnmmBcEJC</t>
+        </is>
+      </c>
       <c r="J728" t="inlineStr"/>
     </row>
     <row r="729">
@@ -29471,7 +29779,7 @@
       </c>
       <c r="E733" t="inlineStr">
         <is>
-          <t>2025/11/19，2025/12/26，2026/03/06</t>
+          <t>2025/11/19，2025/12/26，2026/03/06，2026/08/11</t>
         </is>
       </c>
       <c r="F733" t="inlineStr"/>
@@ -29482,7 +29790,7 @@
       </c>
       <c r="H733" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I733" t="inlineStr">
@@ -29525,7 +29833,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I734" t="inlineStr"/>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>BV1SmBQBdE4b</t>
+        </is>
+      </c>
       <c r="J734" t="inlineStr"/>
     </row>
     <row r="735">
@@ -29623,7 +29935,7 @@
       </c>
       <c r="E737" t="inlineStr">
         <is>
-          <t>2025/11/24</t>
+          <t>2025/11/24，2026/08/02</t>
         </is>
       </c>
       <c r="F737" t="inlineStr"/>
@@ -29634,10 +29946,14 @@
       </c>
       <c r="H737" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I737" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>BV1HbUhByEXN</t>
+        </is>
+      </c>
       <c r="J737" t="inlineStr"/>
     </row>
     <row r="738">
@@ -29743,7 +30059,7 @@
       </c>
       <c r="E740" t="inlineStr">
         <is>
-          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18</t>
+          <t>2025/11/27，2025/11/27，2025/11/28，2025/12/06，2025/12/13，2026/01/10，2026/01/24，2026/02/14，2026/03/14，2026/04/01，2026/04/08，2026/05/01，2026/05/06，2026/05/23，2026/06/20，2026/07/18，2026/08/07</t>
         </is>
       </c>
       <c r="F740" t="inlineStr"/>
@@ -29754,7 +30070,7 @@
       </c>
       <c r="H740" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I740" t="inlineStr">
@@ -29833,7 +30149,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I742" t="inlineStr"/>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>BV14eSwBrEQb</t>
+        </is>
+      </c>
       <c r="J742" t="inlineStr"/>
     </row>
     <row r="743">
@@ -30091,7 +30411,7 @@
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>2025/12/09，2025/12/17，2026/01/14，2026/01/23，2026/02/05，2026/02/10，2026/02/25，2026/04/08，2026/05/01，2026/06/16</t>
+          <t>2025/12/09，2025/12/17，2026/01/14，2026/01/23，2026/02/05，2026/02/10，2026/02/25，2026/04/08，2026/05/01，2026/06/16，2026/8/16</t>
         </is>
       </c>
       <c r="F749" t="inlineStr"/>
@@ -30102,7 +30422,7 @@
       </c>
       <c r="H749" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I749" t="inlineStr">
@@ -30185,7 +30505,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I751" t="inlineStr"/>
+      <c r="I751" t="inlineStr">
+        <is>
+          <t>BV1k9mUB4EG4</t>
+        </is>
+      </c>
       <c r="J751" t="inlineStr"/>
     </row>
     <row r="752">
@@ -30221,7 +30545,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I752" t="inlineStr"/>
+      <c r="I752" t="inlineStr">
+        <is>
+          <t>BV1hNmRBsERE</t>
+        </is>
+      </c>
       <c r="J752" t="inlineStr"/>
     </row>
     <row r="753">
@@ -30257,7 +30585,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I753" t="inlineStr"/>
+      <c r="I753" t="inlineStr">
+        <is>
+          <t>BV13NmRBsEJj</t>
+        </is>
+      </c>
       <c r="J753" t="inlineStr"/>
     </row>
     <row r="754">
@@ -30293,7 +30625,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I754" t="inlineStr"/>
+      <c r="I754" t="inlineStr">
+        <is>
+          <t>BV13NmRBsEED</t>
+        </is>
+      </c>
       <c r="J754" t="inlineStr"/>
     </row>
     <row r="755">
@@ -30423,7 +30759,7 @@
       </c>
       <c r="E758" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/24，2025/12/26，2026/01/02，2026/01/09，2026/01/23，2026/01/29，2026/03/22，2026/04/29，2026/06/20</t>
+          <t>2025/12/19，2025/12/24，2025/12/26，2026/01/02，2026/01/09，2026/01/23，2026/01/29，2026/03/22，2026/04/29，2026/06/20，2026/08/11</t>
         </is>
       </c>
       <c r="F758" t="inlineStr"/>
@@ -30434,7 +30770,7 @@
       </c>
       <c r="H758" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I758" t="inlineStr">
@@ -30539,7 +30875,7 @@
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16</t>
+          <t>2025/12/19，2025/12/23，2025/12/26，2026/01/02，2026/01/05，2026/01/11，2026/01/25，2026/02/09，2026/02/23，2026/03/20，2026/04/02，2026/04/16，2026/04/29，2026/05/10，2026/06/06，2026/06/14，2026/06/20，2026/07/16，2026/08/02，2026/08/07</t>
         </is>
       </c>
       <c r="F761" t="inlineStr"/>
@@ -30550,7 +30886,7 @@
       </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -30579,7 +30915,7 @@
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27</t>
+          <t>2025/12/24，2025/12/24，2025/12/26，2026/01/02，2026/01/10，2026/03/13，2026/06/06，2026/07/09，2026/07/27，2026/08/08</t>
         </is>
       </c>
       <c r="F762" t="inlineStr"/>
@@ -30590,7 +30926,7 @@
       </c>
       <c r="H762" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
@@ -30703,7 +31039,7 @@
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14</t>
+          <t>2025/12/26，2026/01/10，2026/01/22，2026/01/23，2026/01/31，2026/02/10，2026/02/23，2026/03/09，2026/03/12，2026/03/14，2026/03/17，2026/03/27，2026/04/24，2026/05/01，2026/06/14，2026/08/01</t>
         </is>
       </c>
       <c r="F765" t="inlineStr"/>
@@ -30714,7 +31050,7 @@
       </c>
       <c r="H765" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
@@ -31127,7 +31463,7 @@
       </c>
       <c r="E776" t="inlineStr">
         <is>
-          <t>2026/01/24，2026/01/25，2026/01/26，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/03/04，2026/03/12，2026/03/31，2026/04/01，2026/04/14，2026/04/18，2026/05/10，2026/05/23，2026/06/12，2026/07/03，2026/07/21</t>
+          <t>2026/01/24，2026/01/25，2026/01/26，2026/02/02，2026/02/07，2026/02/10，2026/02/14，2026/02/19，2026/03/04，2026/03/12，2026/03/31，2026/04/01，2026/04/14，2026/04/18，2026/05/10，2026/05/23，2026/06/12，2026/07/03，2026/07/21，2026/08/07</t>
         </is>
       </c>
       <c r="F776" t="inlineStr"/>
@@ -31138,7 +31474,7 @@
       </c>
       <c r="H776" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I776" t="inlineStr">
@@ -31411,7 +31747,7 @@
       </c>
       <c r="E783" t="inlineStr">
         <is>
-          <t>2026/02/02，2026/02/05，2026/02/09，2026/02/22，2026/07/25，2026/07/26，2026/07/27</t>
+          <t>2026/02/02，2026/02/05，2026/02/09，2026/02/22，2026/07/25，2026/07/26，2026/07/27，2026/07/31，2026/07/31，2026/08/11</t>
         </is>
       </c>
       <c r="F783" t="inlineStr"/>
@@ -31422,7 +31758,7 @@
       </c>
       <c r="H783" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I783" t="inlineStr">
@@ -31571,7 +31907,7 @@
       </c>
       <c r="E787" t="inlineStr">
         <is>
-          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18</t>
+          <t>2026/02/08，2026/02/09，2026/02/14，2026/02/20，2026/02/28，2026/05/25，2026/06/13，2026/07/05，2026/07/18，2026/08/08</t>
         </is>
       </c>
       <c r="F787" t="inlineStr"/>
@@ -31582,7 +31918,7 @@
       </c>
       <c r="H787" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I787" t="inlineStr">
@@ -31611,7 +31947,7 @@
       </c>
       <c r="E788" t="inlineStr">
         <is>
-          <t>2026/02/08，2026/02/09，2026/02/12，2026/02/14，2026/02/19，2026/02/23，2026/02/24，2026/02/25，2026/03/01，2026/03/05，2026/03/12，2026/03/17，2026/03/19，2026/03/31，2026/04/20，2026/05/02，2026/05/21，2026/06/20，2026/07/16</t>
+          <t>2026/02/08，2026/02/09，2026/02/12，2026/02/14，2026/02/19，2026/02/23，2026/02/24，2026/02/25，2026/03/01，2026/03/05，2026/03/12，2026/03/17，2026/03/19，2026/03/31，2026/04/20，2026/05/02，2026/05/21，2026/06/20，2026/07/16，2026/08/02</t>
         </is>
       </c>
       <c r="F788" t="inlineStr"/>
@@ -31622,7 +31958,7 @@
       </c>
       <c r="H788" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I788" t="inlineStr">
@@ -32019,7 +32355,7 @@
       </c>
       <c r="E798" t="inlineStr">
         <is>
-          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16</t>
+          <t>2026/02/22，2026/02/23，2026/02/24，2026/02/25，2026/03/14，2026/04/20，2026/06/16，2026/08/01</t>
         </is>
       </c>
       <c r="F798" t="inlineStr"/>
@@ -32030,7 +32366,7 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
@@ -32453,7 +32789,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I808" t="inlineStr"/>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>BV17UmJBME1o</t>
+        </is>
+      </c>
       <c r="J808" t="inlineStr"/>
     </row>
     <row r="809">
@@ -32687,7 +33027,7 @@
       </c>
       <c r="E814" t="inlineStr">
         <is>
-          <t>2026/03/13，2026/03/14，2026/03/28，2026/04/29，2026/05/25，2026/06/03，2026/06/13，2026/07/02，2026/07/10，2026/07/15，2026/07/22，2026/07/27</t>
+          <t>2026/03/13，2026/03/14，2026/03/28，2026/04/29，2026/05/25，2026/06/03，2026/06/13，2026/07/02，2026/07/10，2026/07/15，2026/07/22，2026/07/27，2026/07/31，2026/08/11</t>
         </is>
       </c>
       <c r="F814" t="inlineStr"/>
@@ -32698,7 +33038,7 @@
       </c>
       <c r="H814" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I814" t="inlineStr">
@@ -33039,7 +33379,7 @@
       </c>
       <c r="E823" t="inlineStr">
         <is>
-          <t>2026/03/17，2026/03/17，2026/03/25，2026/03/27，2026/03/29，2026/04/02，2026/04/08，2026/04/16，2026/04/20，2026/05/02，2026/05/06，2026/05/26，2026/06/14，2026/07/18</t>
+          <t>2026/03/17，2026/03/17，2026/03/25，2026/03/27，2026/03/29，2026/04/02，2026/04/08，2026/04/16，2026/04/20，2026/05/02，2026/05/06，2026/05/26，2026/06/14，2026/07/18，2026/08/08</t>
         </is>
       </c>
       <c r="F823" t="inlineStr"/>
@@ -33050,7 +33390,7 @@
       </c>
       <c r="H823" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I823" t="inlineStr">
@@ -33135,7 +33475,7 @@
       </c>
       <c r="E825" t="inlineStr">
         <is>
-          <t>2026/03/25，2026/04/14，2026/05/25，2026/05/25，2026/06/25，2026/06/25，2026/06/25，2026/06/26，2026/07/07</t>
+          <t>2026/03/25，2026/04/14，2026/05/25，2026/05/25，2026/06/25，2026/06/25，2026/06/25，2026/06/26，2026/07/07，2026/08/09</t>
         </is>
       </c>
       <c r="F825" t="inlineStr"/>
@@ -33146,7 +33486,7 @@
       </c>
       <c r="H825" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I825" t="inlineStr">
@@ -33837,7 +34177,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I842" t="inlineStr"/>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>BV1PEQVBuEKU</t>
+        </is>
+      </c>
       <c r="J842" t="inlineStr"/>
     </row>
     <row r="843">
@@ -33939,7 +34283,7 @@
       </c>
       <c r="E845" t="inlineStr">
         <is>
-          <t>2026/04/17，2026/05/25，2026/05/25，2026/05/26</t>
+          <t>2026/04/17，2026/05/25，2026/05/25，2026/05/26，2026/08/02</t>
         </is>
       </c>
       <c r="F845" t="inlineStr"/>
@@ -33950,7 +34294,7 @@
       </c>
       <c r="H845" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I845" t="inlineStr">
@@ -34041,7 +34385,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I847" t="inlineStr"/>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>BV1UodkBzE3C</t>
+        </is>
+      </c>
       <c r="J847" t="inlineStr"/>
     </row>
     <row r="848">
@@ -34235,7 +34583,7 @@
       </c>
       <c r="E852" t="inlineStr">
         <is>
-          <t>2026/05/01</t>
+          <t>2026/05/01，2026/07/31，2026/08/01，2026/08/08，2026/08/11</t>
         </is>
       </c>
       <c r="F852" t="inlineStr"/>
@@ -34246,7 +34594,7 @@
       </c>
       <c r="H852" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I852" t="inlineStr">
@@ -34315,7 +34663,7 @@
       </c>
       <c r="E854" t="inlineStr">
         <is>
-          <t>2026/05/01</t>
+          <t>2026/05/01，2026/08/02</t>
         </is>
       </c>
       <c r="F854" t="inlineStr"/>
@@ -34326,7 +34674,7 @@
       </c>
       <c r="H854" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I854" t="inlineStr">
@@ -34575,7 +34923,7 @@
       </c>
       <c r="E860" t="inlineStr">
         <is>
-          <t>2026/05/25，2026/05/26，2026/06/15</t>
+          <t>2026/05/25，2026/05/26，2026/06/15，2026/08/02</t>
         </is>
       </c>
       <c r="F860" t="inlineStr"/>
@@ -34586,7 +34934,7 @@
       </c>
       <c r="H860" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I860" t="inlineStr">
@@ -34815,7 +35163,7 @@
       </c>
       <c r="E866" t="inlineStr">
         <is>
-          <t>2026/06/14，2026/06/14</t>
+          <t>2026/06/14，2026/06/14，2026/08/02</t>
         </is>
       </c>
       <c r="F866" t="inlineStr"/>
@@ -34826,7 +35174,7 @@
       </c>
       <c r="H866" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I866" t="inlineStr">
@@ -35037,7 +35385,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I871" t="inlineStr"/>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>BV1XGjb6yEbo</t>
+        </is>
+      </c>
       <c r="J871" t="inlineStr"/>
     </row>
     <row r="872">
@@ -35099,7 +35451,7 @@
       </c>
       <c r="E873" t="inlineStr">
         <is>
-          <t>2026/06/25，2026/07/09，2026/07/18</t>
+          <t>2026/06/25，2026/07/09，2026/07/18，2026/07/31</t>
         </is>
       </c>
       <c r="F873" t="inlineStr"/>
@@ -35110,7 +35462,7 @@
       </c>
       <c r="H873" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I873" t="inlineStr">
@@ -35139,7 +35491,7 @@
       </c>
       <c r="E874" t="inlineStr">
         <is>
-          <t>2026/06/25</t>
+          <t>2026/06/25，2026/08/01，2026/08/11</t>
         </is>
       </c>
       <c r="F874" t="inlineStr"/>
@@ -35150,7 +35502,7 @@
       </c>
       <c r="H874" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I874" t="inlineStr">
@@ -35263,7 +35615,7 @@
       </c>
       <c r="E877" t="inlineStr">
         <is>
-          <t>2026/07/07，2026/07/09，2026/07/10，2026/07/15，2026/07/16，2026/07/18，2026/07/25，2026/07/27</t>
+          <t>2026/07/07，2026/07/09，2026/07/10，2026/07/15，2026/07/16，2026/07/18，2026/07/25，2026/07/27，2026/08/01，2026/08/08，2026/08/11</t>
         </is>
       </c>
       <c r="F877" t="inlineStr"/>
@@ -35274,7 +35626,7 @@
       </c>
       <c r="H877" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I877" t="inlineStr">
@@ -35303,7 +35655,7 @@
       </c>
       <c r="E878" t="inlineStr">
         <is>
-          <t>2026/07/17，2026/07/18，2026/07/27</t>
+          <t>2026/07/17，2026/07/18，2026/07/27，2026/08/02，2026/08/05</t>
         </is>
       </c>
       <c r="F878" t="inlineStr"/>
@@ -35314,7 +35666,7 @@
       </c>
       <c r="H878" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I878" t="inlineStr">
@@ -35383,7 +35735,7 @@
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>2026/07/26，2026/07/27，2026/07/28</t>
+          <t>2026/07/26，2026/07/27，2026/07/28，2026/07/31，2026/07/31，2026/08/08</t>
         </is>
       </c>
       <c r="F880" t="inlineStr"/>
@@ -35394,7 +35746,7 @@
       </c>
       <c r="H880" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I880" t="inlineStr">
@@ -35423,7 +35775,7 @@
       </c>
       <c r="E881" t="inlineStr">
         <is>
-          <t>2026/07/27</t>
+          <t>2026/07/27，2026/07/30，2026/08/01，2026/08/03</t>
         </is>
       </c>
       <c r="F881" t="inlineStr"/>
@@ -35434,7 +35786,7 @@
       </c>
       <c r="H881" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I881" t="inlineStr">
@@ -35503,7 +35855,7 @@
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>2026/07/27</t>
+          <t>2026/07/27，2026/07/31</t>
         </is>
       </c>
       <c r="F883" t="inlineStr"/>
@@ -35514,15 +35866,247 @@
       </c>
       <c r="H883" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>BV19x3P6cESt</t>
+        </is>
+      </c>
+      <c r="J883" t="inlineStr"/>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>883</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>蝴蝶泉边</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr"/>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>黄雅莉</t>
+        </is>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>2026/08/02</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr"/>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I883" t="inlineStr">
-        <is>
-          <t>BV19x3P6cESt</t>
-        </is>
-      </c>
-      <c r="J883" t="inlineStr"/>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>BV1Qm3Z61Exc</t>
+        </is>
+      </c>
+      <c r="J884" t="inlineStr"/>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>884</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>麦恩莉</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr"/>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>方大同</t>
+        </is>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>2026/08/03，2026/08/08，2026/08/09，2026/08/11</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr"/>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>BV1BTMo6VELH</t>
+        </is>
+      </c>
+      <c r="J885" t="inlineStr"/>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>885</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>中国人会飞</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr"/>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Chalky Wong/揽佬SKAI ISYOURGOD</t>
+        </is>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>2026/08/05，2026/08/05</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr"/>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>BV1cZMy6DE4V</t>
+        </is>
+      </c>
+      <c r="J886" t="inlineStr"/>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>886</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Enemy</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr"/>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>Imagine Dragons/JID/英雄联盟/双城之战</t>
+        </is>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>2026/08/05，2025/05/03</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr"/>
+      <c r="G887" t="inlineStr">
+        <is>
+          <t>英语</t>
+        </is>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>BV1scGdzVEjo</t>
+        </is>
+      </c>
+      <c r="J887" t="inlineStr"/>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>887</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>悲伤的五个步骤</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr"/>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>艾薇Ivy</t>
+        </is>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>2026/08/11，2026/08/11</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr"/>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr"/>
+      <c r="J888" t="inlineStr"/>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>讨厌</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr"/>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>芮恩</t>
+        </is>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>2026/08/11</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr"/>
+      <c r="G889" t="inlineStr">
+        <is>
+          <t>华语</t>
+        </is>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr"/>
+      <c r="J889" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>